<commit_message>
Clarify investment project roadmap and stress workflow
</commit_message>
<xml_diff>
--- a/files/BUS331_InvProject_StressTest_Template.xlsx
+++ b/files/BUS331_InvProject_StressTest_Template.xlsx
@@ -2,11 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="START HERE" sheetId="1" r:id="R849daad805a44a35"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SUMMARY" sheetId="2" r:id="Racac44fdfb9244b4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client 1" sheetId="3" r:id="R8015c8792fae4d71"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client 2" sheetId="4" r:id="R84dd12c81d10406c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client 3" sheetId="5" r:id="Raab37177514948af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="START HERE" sheetId="1" r:id="Ra751a2d8d3f145a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SUMMARY" sheetId="2" r:id="R9c5763a73c8f44e1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client 1" sheetId="3" r:id="Rd5fb0cd4e101492c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client 2" sheetId="4" r:id="R5ef4c4ca42eb409b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client 3" sheetId="5" r:id="Rabe819069bf94e0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SCENARIO REVEAL" sheetId="6" r:id="R268ff1a878c544d5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1958,46 +1959,7 @@
     <x:t xml:space="preserve">Student Workbook  |  Endicott College  |  Institutional Portfolio Management Project</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">  Overview — 5 Tabs</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">This workbook has five tabs: START HERE, SUMMARY, Client 1, Client 2, Client 3.
-Complete one client tab for each of your three assigned clients.
-The SUMMARY tab auto-links key results from all three client tabs.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">  Before You Start</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">  Section 1 — Bear Case Scenario Assumptions</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Enter your Phase 1 Bear Case expected returns and standard deviations for each asset class (equities, fixed income, cash). These MUST match your Phase 1 submission exactly — do not adjust them here. Cite your Phase 1 source in the rightmost column.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">  Section 2 — Base Case Portfolio</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">  Section 3 — Risk Metrics</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">  Section 4 — Pass / Fail Verdict</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">The workbook automatically compares your Bear Case portfolio return to the IPS Tripwire. GREEN = PASS: portfolio survives the Bear Case within the client's drawdown limit.
-RED = FAIL: portfolio breaches the mandate — you must complete Section 5.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">  Section 5 — Re-allocation (FAIL only)</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">If a client fails, document the specific trades in Part A: what was sold, what was bought, old and new weights, dollar impact, and rationale. Part B re-runs the Bear Case with the new weights. The revised verdict must be PASS before submitting.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">  Section 6 — Final Metrics Summary</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Enter the final metrics for submission: β, σ, Sharpe, Bear Case return, dollar P&amp;L, and mandate status. Use revised figures if you re-allocated in Section 5.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">  AI Audit Log Reminder</x:t>
@@ -2007,36 +1969,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">  PRE-SUBMISSION CHECKLIST</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">☐  Bear Case assumptions match Phase 1 Bear Case scenario table exactly</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">☐  Portfolio weights sum to 100% in Section 2 (total cell is green)</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">☐  Risk-Free Rate (Rf) entered in Section 3</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">☐  Beta and σ entered for both Base Case and Bear Case</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">☐  Section 4 verdict calculated for all three clients</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">☐  Section 5 re-allocation completed for any client that failed</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">☐  Revised verdict in Section 5 shows PASS for all re-allocated clients</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">☐  Section 6 final metrics entered and reflect re-allocation if applicable</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">☐  SUMMARY tab shows all three clients passing before team submits</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">☐  AI Audit Log updated for any AI-assisted analysis</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">BUS 331 Investments  |  Endicott College  |  Cross-client Comparison</x:t>
@@ -2057,15 +1989,6 @@
     <x:t xml:space="preserve">IPS Tripwire (max drawdown)</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Bear Case Portfolio Return</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Bear Case $ P&amp;L ($500K AUM)</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Section 4 Verdict (Pass/Fail)</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Portfolio Beta (β)</x:t>
   </x:si>
   <x:si>
@@ -2073,9 +1996,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Sharpe Ratio — Base Case</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Re-allocation Required?</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Client Name / ID:</x:t>
@@ -2093,26 +2013,6 @@
     <x:t xml:space="preserve">(from Phase 2)</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">  SECTION 1 — BEAR CASE SCENARIO ASSUMPTIONS  (from Phase 1)</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Enter your Phase 1 Bear Case return assumptions for each asset class. These must match your Phase 1 submission exactly — do not change them here. Source: your team's Phase 1 Bear Case scenario table.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Asset Class</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Bear Case
-E(R) Assumption</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Bear Case
-Std Dev (σ)</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Source / Phase 1 Reference</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">U.S. Equities</x:t>
   </x:si>
   <x:si>
@@ -2122,20 +2022,11 @@
     <x:t xml:space="preserve">Cash / Cash Equivalents</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">Asset Class</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">$ Allocation
 ($500K AUM)</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Base Case
-E(R) Contrib.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Bear Case
-Return Contrib.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Bear Case
-$ P&amp;L</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Notes</x:t>
@@ -2145,15 +2036,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">  PORTFOLIO TOTAL</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">  ← Bear Case return must be ≥ IPS Tripwire (cell G5). See Section 3 verdict below.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">  SECTION 3 — RISK METRICS  (Base Case &amp; Bear Case)</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Bear Case</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Formula / Source</x:t>
@@ -2186,16 +2068,7 @@
     <x:t xml:space="preserve">Higher = better risk-adjusted return; compare Base vs Bear to see deterioration</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Max Drawdown (Bear Case)</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">N/A</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Total Bear Case Portfolio Return (Section 2 row 20)</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Must be ≥ IPS Tripwire (cell G5). This drives the Pass/Fail verdict.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Value at Risk — 95% VaR</x:t>
@@ -2205,9 +2078,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">There is a 5% chance of loss worse than this. Compare to IPS Tripwire.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">  SECTION 4 — PASS / FAIL VERDICT</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Test</x:t>
@@ -2233,12 +2103,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">If σ exceeds IPS limit, consider adding cash or fixed income to reduce volatility.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">  SECTION 5 — RE-ALLOCATION  (complete only if Section 4 verdict = FAIL)</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">If the portfolio failed the Tripwire, document the specific trades made to bring it within mandate. Describe what was sold, what was bought, the new weights, and show the re-run stress test confirms the revised portfolio now PASSES.</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">  Part A — Trade Log  (specific securities sold / bought)</x:t>
@@ -2269,22 +2133,10 @@
     <x:t xml:space="preserve">← Must equal 100% after re-allocation</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">  Part B — Revised Bear Case Return  (confirm portfolio now PASSES)</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Using your new weights from Part A, recalculate the Bear Case portfolio return. The result must be ≥ the IPS Tripwire. Show your calculation clearly.</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">NEW Weight</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">$ Allocation</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Bear Case E(R)</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Wtd Bear Contribution</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">$ P&amp;L</x:t>
@@ -2294,12 +2146,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">REVISED VERDICT:</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Revised Bear Case return must be ≥ IPS Tripwire (G5). If still failing, increase cash allocation or add a derivative hedge.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">  SECTION 6 — FINAL RISK METRICS SUMMARY  (for submission)</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Final Value</x:t>
@@ -2329,13 +2175,7 @@
     <x:t xml:space="preserve">From Section 2 total row (or Section 5 revised total if re-allocated)</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Bear Case $ P&amp;L</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Dollar impact on $500K AUM</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">IPS Mandate Status</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Final verdict for this client</x:t>
@@ -2380,7 +2220,7 @@
     <x:numFmt numFmtId="168" formatCode="\$#,##0"/>
     <x:numFmt numFmtId="169" formatCode="0.0"/>
   </x:numFmts>
-  <x:fonts count="27">
+  <x:fonts count="33">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -2522,8 +2362,42 @@
       <x:sz val="10"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="16"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF516173"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="12"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF263746"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="9"/>
+      <x:color rgb="FF0B1C33"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF1F5D95"/>
+      <x:name val="Calibri"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="12">
+  <x:fills count="16">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -2580,8 +2454,28 @@
         <x:fgColor rgb="FFD4EDDA"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0B1C33"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF3FB"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFDDE9F3"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF4D6"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="18">
+  <x:borders count="31">
     <x:border diagonalUp="0" diagonalDown="0"/>
     <x:border diagonalUp="0" diagonalDown="0">
       <x:bottom style="medium">
@@ -2740,6 +2634,116 @@
         <x:color rgb="FFC9A84C"/>
       </x:top>
     </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="medium">
+        <x:color rgb="FFD59A22"/>
+      </x:left>
+      <x:top style="medium">
+        <x:color rgb="FFD59A22"/>
+      </x:top>
+      <x:bottom style="medium">
+        <x:color rgb="FFD59A22"/>
+      </x:bottom>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:top style="medium">
+        <x:color rgb="FFD59A22"/>
+      </x:top>
+      <x:bottom style="medium">
+        <x:color rgb="FFD59A22"/>
+      </x:bottom>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:right style="medium">
+        <x:color rgb="FFD59A22"/>
+      </x:right>
+      <x:top style="medium">
+        <x:color rgb="FFD59A22"/>
+      </x:top>
+      <x:bottom style="medium">
+        <x:color rgb="FFD59A22"/>
+      </x:bottom>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="thin">
+        <x:color rgb="FFB7C9DA"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FFB7C9DA"/>
+      </x:top>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:top style="thin">
+        <x:color rgb="FFB7C9DA"/>
+      </x:top>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:right style="thin">
+        <x:color rgb="FFB7C9DA"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFB7C9DA"/>
+      </x:top>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="thin">
+        <x:color rgb="FFB7C9DA"/>
+      </x:left>
+      <x:bottom style="thin">
+        <x:color rgb="FFB7C9DA"/>
+      </x:bottom>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:bottom style="thin">
+        <x:color rgb="FFB7C9DA"/>
+      </x:bottom>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:right style="thin">
+        <x:color rgb="FFB7C9DA"/>
+      </x:right>
+      <x:bottom style="thin">
+        <x:color rgb="FFB7C9DA"/>
+      </x:bottom>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="thin">
+        <x:color rgb="FFB7C9DA"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFB7C9DA"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFB7C9DA"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFB7C9DA"/>
+      </x:bottom>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="thin">
+        <x:color rgb="FFB7C9DA"/>
+      </x:left>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:right style="thin">
+        <x:color rgb="FFB7C9DA"/>
+      </x:right>
+    </x:border>
+    <x:border diagonalUp="0" diagonalDown="0">
+      <x:left style="thin">
+        <x:color rgb="FFD59A22"/>
+      </x:left>
+      <x:right style="thin">
+        <x:color rgb="FFD59A22"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FFD59A22"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD59A22"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="20">
     <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -2766,7 +2770,7 @@
     <x:xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <x:xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="64">
+  <x:cellXfs count="100">
     <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="0" applyBorder="0" applyAlignment="0">
       <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
     </x:xf>
@@ -2958,6 +2962,114 @@
     </x:xf>
     <x:xf numFmtId="164" fontId="15" fillId="8" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="27" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="27" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="28" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="29" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="29" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="29" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="29" fillId="12" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="29" fillId="12" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="29" fillId="12" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="30" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="30" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="30" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="30" fillId="13" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="30" fillId="13" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="30" fillId="13" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="30" fillId="13" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="30" fillId="13" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="30" fillId="13" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="31" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="31" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="31" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="31" fillId="14" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="32" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="30" fillId="13" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="30" fillId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="0" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="30" fillId="13" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="31" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="31" fillId="15" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="6">
@@ -3323,59 +3435,56 @@
     </x:row>
     <x:row r="4" ht="7.5" hidden="0" customHeight="1"/>
     <x:row r="5" ht="19.5" hidden="0" customHeight="1">
-      <x:c r="B5" s="4" t="s">
-        <x:v>1</x:v>
+      <x:c r="B5" s="4" t="str">
+        <x:v>  Overview — 6 Tabs</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="51.75" hidden="0" customHeight="1">
-      <x:c r="B6" s="5" t="s">
-        <x:v>2</x:v>
+      <x:c r="B6" s="5" t="str">
+        <x:v>This workbook has six tabs: START HERE, SUMMARY, Client 1, Client 2, Client 3, and SCENARIO REVEAL. Complete one client tab for each assigned client. The SUMMARY tab auto-links key results; use SCENARIO REVEAL only after the instructor releases the adverse-event packet.</x:v>
       </x:c>
       <x:c r="C6" s="5"/>
     </x:row>
     <x:row r="7" ht="7.5" hidden="0" customHeight="1"/>
     <x:row r="8" ht="19.5" hidden="0" customHeight="1">
-      <x:c r="B8" s="4" t="s">
-        <x:v>3</x:v>
+      <x:c r="B8" s="4" t="str">
+        <x:v>  Two-stage workflow — baseline, then Scenario Reveal</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="51.75" hidden="0" customHeight="1">
       <x:c r="B9" s="5" t="str">
-        <x:v>Before opening a client tab, confirm three inputs:
-• Phase 1: Approved Bear Case E(R) and σ assumptions for each asset class
-• Phase 1: Each client's IPS Tripwire, max σ, and other relevant guardrails
-• Phase 2 Workstreams A and B: Solver-supported weights, selected holdings, β, σ, and Sharpe Ratio</x:v>
+        <x:v>Stage 1: Build and submit the baseline portfolio snapshot using the approved Phase 1 bear-case inputs and client guardrails. Stage 2: After the baseline checkpoint, record the instructor-issued Scenario Reveal, transfer its exact inputs to each Client tab, test the result, document a required corrective trade for each breach, and re-test before Gate 2.</x:v>
       </x:c>
       <x:c r="C9" s="5"/>
     </x:row>
     <x:row r="10" ht="7.5" hidden="0" customHeight="1"/>
     <x:row r="11" ht="19.5" hidden="0" customHeight="1">
-      <x:c r="B11" s="4" t="s">
-        <x:v>4</x:v>
+      <x:c r="B11" s="4" t="str">
+        <x:v>  Section 1 — Scenario Reveal Assumptions</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="51.75" hidden="0" customHeight="1">
-      <x:c r="B12" s="5" t="s">
-        <x:v>5</x:v>
+      <x:c r="B12" s="5" t="str">
+        <x:v>After the baseline checkpoint, enter the instructor-issued scenario inputs exactly as released. They replace the initial scenario inputs only for the remediation test. Record the packet ID and release date on SCENARIO REVEAL; do not change the mandate, soften the scenario, or invent values.</x:v>
       </x:c>
       <x:c r="C12" s="5"/>
     </x:row>
     <x:row r="13" ht="7.5" hidden="0" customHeight="1"/>
     <x:row r="14" ht="19.5" hidden="0" customHeight="1">
-      <x:c r="B14" s="4" t="s">
-        <x:v>6</x:v>
+      <x:c r="B14" s="4" t="str">
+        <x:v>  Section 2 — Baseline Portfolio</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="51.75" hidden="0" customHeight="1">
       <x:c r="B15" s="5" t="str">
-        <x:v>Enter the Workstream A Solver-supported weights for each asset class. Also enter the Base Case E(R) for each class from the Phase 2 CME Matrix. Bear Case return contributions and dollar P&amp;L calculate automatically.</x:v>
+        <x:v>Enter the submitted baseline weights from Workstream A. Keep the original allocation in the Canvas baseline snapshot. After the Scenario Reveal, use Section 5 to document the actual changes and the complete re-test.</x:v>
       </x:c>
       <x:c r="C15" s="5"/>
     </x:row>
     <x:row r="16" ht="7.5" hidden="0" customHeight="1"/>
     <x:row r="17" ht="19.5" hidden="0" customHeight="1">
       <x:c r="B17" s="4" t="s">
-        <x:v>7</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="51.75" hidden="0" customHeight="1">
@@ -3386,114 +3495,114 @@
     </x:row>
     <x:row r="19" ht="7.5" hidden="0" customHeight="1"/>
     <x:row r="20" ht="19.5" hidden="0" customHeight="1">
-      <x:c r="B20" s="4" t="s">
-        <x:v>8</x:v>
+      <x:c r="B20" s="4" t="str">
+        <x:v>  Section 4 — Scenario Reveal Verdict</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="51.75" hidden="0" customHeight="1">
-      <x:c r="B21" s="5" t="s">
-        <x:v>9</x:v>
+      <x:c r="B21" s="5" t="str">
+        <x:v>The workbook compares the revealed-scenario portfolio return with the IPS Tripwire. GREEN = PASS; RED = BREACH. A Scenario Reveal packet is calibrated to generate a meaningful decision. If your result is PASS, notify the instructor rather than skipping the remediation checkpoint.</x:v>
       </x:c>
       <x:c r="C21" s="5"/>
     </x:row>
     <x:row r="22" ht="7.5" hidden="0" customHeight="1"/>
     <x:row r="23" ht="19.5" hidden="0" customHeight="1">
-      <x:c r="B23" s="4" t="s">
-        <x:v>10</x:v>
+      <x:c r="B23" s="4" t="str">
+        <x:v>  Section 5 — Required Remediation &amp; Re-test</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="51.75" hidden="0" customHeight="1">
-      <x:c r="B24" s="5" t="s">
-        <x:v>11</x:v>
+      <x:c r="B24" s="5" t="str">
+        <x:v>For every Scenario Reveal breach, document the specific trades: what was sold, what was bought, old and new weights, dollar impact, rationale, and client trade-off. Re-run the full scenario and IPS tests. A narrative alone does not cure a breach.</x:v>
       </x:c>
       <x:c r="C24" s="5"/>
     </x:row>
     <x:row r="25" ht="7.5" hidden="0" customHeight="1"/>
     <x:row r="26" ht="19.5" hidden="0" customHeight="1">
-      <x:c r="B26" s="4" t="s">
-        <x:v>12</x:v>
+      <x:c r="B26" s="4" t="str">
+        <x:v>  Section 6 — Final Metrics Summary</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="51.75" hidden="0" customHeight="1">
-      <x:c r="B27" s="5" t="s">
-        <x:v>13</x:v>
+      <x:c r="B27" s="5" t="str">
+        <x:v>Enter the final metrics for Gate 2: beta, standard deviation, Sharpe, Scenario Reveal return, dollar P&amp;L, and mandate status. Use the revised figures after remediation and retain the baseline evidence separately.</x:v>
       </x:c>
       <x:c r="C27" s="5"/>
     </x:row>
     <x:row r="28" ht="7.5" hidden="0" customHeight="1"/>
     <x:row r="29" ht="19.5" hidden="0" customHeight="1">
       <x:c r="B29" s="4" t="s">
-        <x:v>14</x:v>
+        <x:v>2</x:v>
       </x:c>
     </x:row>
     <x:row r="30" ht="51.75" hidden="0" customHeight="1">
       <x:c r="B30" s="5" t="s">
-        <x:v>15</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="C30" s="5"/>
     </x:row>
     <x:row r="32" ht="19.5" hidden="0" customHeight="1">
       <x:c r="B32" s="6" t="s">
-        <x:v>16</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="33" ht="18" hidden="0" customHeight="1">
-      <x:c r="B33" s="7" t="s">
-        <x:v>17</x:v>
+      <x:c r="B33" s="7" t="str">
+        <x:v>☐  Baseline allocation, IPS scorecard, and initial results submitted before Scenario Reveal</x:v>
       </x:c>
       <x:c r="C33" s="7"/>
     </x:row>
     <x:row r="34" ht="18" hidden="0" customHeight="1">
-      <x:c r="B34" s="7" t="s">
-        <x:v>18</x:v>
+      <x:c r="B34" s="7" t="str">
+        <x:v>☐  Scenario Release Log completed with packet ID, date, client condition tested, and Canvas receipt</x:v>
       </x:c>
       <x:c r="C34" s="7"/>
     </x:row>
     <x:row r="35" ht="18" hidden="0" customHeight="1">
-      <x:c r="B35" s="7" t="s">
-        <x:v>19</x:v>
+      <x:c r="B35" s="7" t="str">
+        <x:v>☐  Released scenario inputs copied exactly; mandate and tripwire unchanged</x:v>
       </x:c>
       <x:c r="C35" s="7"/>
     </x:row>
     <x:row r="36" ht="18" hidden="0" customHeight="1">
-      <x:c r="B36" s="7" t="s">
-        <x:v>20</x:v>
+      <x:c r="B36" s="7" t="str">
+        <x:v>☐  Portfolio weights sum to 100% in the baseline and revised allocation</x:v>
       </x:c>
       <x:c r="C36" s="7"/>
     </x:row>
     <x:row r="37" ht="18" hidden="0" customHeight="1">
-      <x:c r="B37" s="7" t="s">
-        <x:v>21</x:v>
+      <x:c r="B37" s="7" t="str">
+        <x:v>☐  Risk-Free Rate (Rf), beta, and standard deviation entered with sources</x:v>
       </x:c>
       <x:c r="C37" s="7"/>
     </x:row>
     <x:row r="38" ht="18" hidden="0" customHeight="1">
-      <x:c r="B38" s="7" t="s">
-        <x:v>22</x:v>
+      <x:c r="B38" s="7" t="str">
+        <x:v>☐  Scenario Reveal verdict calculated for all three clients</x:v>
       </x:c>
       <x:c r="C38" s="7"/>
     </x:row>
     <x:row r="39" ht="18" hidden="0" customHeight="1">
-      <x:c r="B39" s="7" t="s">
-        <x:v>23</x:v>
+      <x:c r="B39" s="7" t="str">
+        <x:v>☐  Every breach has a documented security, sleeve, or weight change and trade-off</x:v>
       </x:c>
       <x:c r="C39" s="7"/>
     </x:row>
     <x:row r="40" ht="18" hidden="0" customHeight="1">
-      <x:c r="B40" s="7" t="s">
-        <x:v>24</x:v>
+      <x:c r="B40" s="7" t="str">
+        <x:v>☐  Revised scenario and full IPS scorecard re-tested after each corrective trade</x:v>
       </x:c>
       <x:c r="C40" s="7"/>
     </x:row>
     <x:row r="41" ht="18" hidden="0" customHeight="1">
-      <x:c r="B41" s="7" t="s">
-        <x:v>25</x:v>
+      <x:c r="B41" s="7" t="str">
+        <x:v>☐  SUMMARY tab shows final Gate 2 results and the committee has recorded its vote</x:v>
       </x:c>
       <x:c r="C41" s="7"/>
     </x:row>
     <x:row r="42" ht="18" hidden="0" customHeight="1">
-      <x:c r="B42" s="7" t="s">
-        <x:v>26</x:v>
+      <x:c r="B42" s="7" t="str">
+        <x:v>☐  AI Audit Log updated for any AI-assisted analysis</x:v>
       </x:c>
       <x:c r="C42" s="7"/>
     </x:row>
@@ -3541,7 +3650,7 @@
     <x:row r="1" ht="6" hidden="0" customHeight="1"/>
     <x:row r="2" ht="37.5" hidden="0" customHeight="1">
       <x:c r="A2" s="2" t="str">
-        <x:v>Phase 2 Workstream C — Portfolio Stress Test Summary — All Clients</x:v>
+        <x:v>Phase 2 Workstream C — Scenario Reveal &amp; Remediation Summary — All Clients</x:v>
       </x:c>
       <x:c r="B2" s="2"/>
       <x:c r="C2" s="2"/>
@@ -3551,7 +3660,7 @@
     </x:row>
     <x:row r="3" ht="18" hidden="0" customHeight="1">
       <x:c r="A3" s="3" t="s">
-        <x:v>27</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="B3" s="3"/>
       <x:c r="C3" s="3"/>
@@ -3561,7 +3670,7 @@
     </x:row>
     <x:row r="4" ht="31.5" hidden="0" customHeight="1">
       <x:c r="A4" s="8" t="str">
-        <x:v>This tab auto-links key stress-test results from each client tab. All three clients must satisfy the tripwire and complete the full IPS scorecard before the Phase 2 committee vote.</x:v>
+        <x:v>This tab links the revealed-scenario results from each client tab. Keep the separate Canvas baseline snapshot; this workbook documents the instructor-issued Scenario Reveal, corrective trades, and re-test required for Gate 2.</x:v>
       </x:c>
       <x:c r="B4" s="8"/>
       <x:c r="C4" s="8"/>
@@ -3572,21 +3681,21 @@
     <x:row r="5" ht="7.5" hidden="0" customHeight="1"/>
     <x:row r="6" ht="30" hidden="0" customHeight="1">
       <x:c r="B6" s="9" t="s">
-        <x:v>28</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C6" s="9" t="s">
-        <x:v>29</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="D6" s="9" t="s">
-        <x:v>30</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="E6" s="9" t="s">
-        <x:v>31</x:v>
+        <x:v>9</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="25.5" hidden="0" customHeight="1">
       <x:c r="B7" s="10" t="s">
-        <x:v>32</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C7" s="11" t="n">
         <x:f aca="0">'Client 1'!G5</x:f>
@@ -3602,8 +3711,8 @@
       </x:c>
     </x:row>
     <x:row r="8" ht="25.5" hidden="0" customHeight="1">
-      <x:c r="B8" s="12" t="s">
-        <x:v>33</x:v>
+      <x:c r="B8" s="12" t="str">
+        <x:v>Scenario Reveal Portfolio Return</x:v>
       </x:c>
       <x:c r="C8" s="11" t="n">
         <x:f aca="0">'Client 1'!F20</x:f>
@@ -3619,8 +3728,8 @@
       </x:c>
     </x:row>
     <x:row r="9" ht="25.5" hidden="0" customHeight="1">
-      <x:c r="B9" s="10" t="s">
-        <x:v>34</x:v>
+      <x:c r="B9" s="10" t="str">
+        <x:v>Scenario Reveal $ P&amp;L ($500K AUM)</x:v>
       </x:c>
       <x:c r="C9" s="13" t="n">
         <x:f aca="0">'Client 1'!G20</x:f>
@@ -3636,8 +3745,8 @@
       </x:c>
     </x:row>
     <x:row r="10" ht="25.5" hidden="0" customHeight="1">
-      <x:c r="B10" s="12" t="s">
-        <x:v>35</x:v>
+      <x:c r="B10" s="12" t="str">
+        <x:v>Scenario Reveal Verdict (Pass / Breach)</x:v>
       </x:c>
       <x:c r="C10" s="14" t="str">
         <x:f aca="0">'Client 1'!F34</x:f>
@@ -3651,7 +3760,7 @@
     </x:row>
     <x:row r="11" ht="25.5" hidden="0" customHeight="1">
       <x:c r="B11" s="10" t="s">
-        <x:v>36</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C11" s="15" t="n">
         <x:f aca="0">'Client 1'!C26</x:f>
@@ -3668,7 +3777,7 @@
     </x:row>
     <x:row r="12" ht="25.5" hidden="0" customHeight="1">
       <x:c r="B12" s="12" t="s">
-        <x:v>37</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="C12" s="11" t="n">
         <x:f aca="0">'Client 1'!C27</x:f>
@@ -3685,7 +3794,7 @@
     </x:row>
     <x:row r="13" ht="25.5" hidden="0" customHeight="1">
       <x:c r="B13" s="10" t="s">
-        <x:v>38</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="C13" s="15" t="str">
         <x:f aca="0">'Client 1'!C28</x:f>
@@ -3698,8 +3807,8 @@
       </x:c>
     </x:row>
     <x:row r="14" ht="25.5" hidden="0" customHeight="1">
-      <x:c r="B14" s="12" t="s">
-        <x:v>39</x:v>
+      <x:c r="B14" s="12" t="str">
+        <x:v>Remediation &amp; re-test required?</x:v>
       </x:c>
       <x:c r="C14" s="14" t="str">
         <x:f aca="0">IF('Client 1'!F34="","",IF('Client 1'!F34="✓ PASS","NO","YES"))</x:f>
@@ -3714,8 +3823,8 @@
     <x:row r="16" ht="7.5" hidden="0" customHeight="1"/>
     <x:row r="17" ht="30" hidden="0" customHeight="1">
       <x:c r="A17" s="16" t="str">
-        <x:f aca="0">IF(AND('Client 1'!F34="✓ PASS",'Client 2'!F34="✓ PASS",'Client 3'!F34="✓ PASS"),"  ✓ ALL THREE CLIENTS PASS — Ready for the Phase 2 committee vote and Phase 3 defense","  ✗ ONE OR MORE CLIENTS FAILING — Complete Section 5 re-allocation and re-test before approval")</x:f>
-        <x:v>  ✗ ONE OR MORE CLIENTS FAILING — Complete Section 5 re-allocation and re-test before approval</x:v>
+        <x:f aca="0">IF(AND('Client 1'!F56="✓ REVISED PASS",'Client 2'!F56="✓ REVISED PASS",'Client 3'!F56="✓ REVISED PASS"),"  ✓ ALL THREE CLIENTS REMEDIATED AND RE-TESTED — Ready for the Phase 2 committee vote","  ✗ ONE OR MORE CLIENTS STILL NEEDS REMEDIATION OR RE-TESTING — Do not approve Gate 2")</x:f>
+        <x:v>  ✗ ONE OR MORE CLIENTS STILL NEEDS REMEDIATION OR RE-TESTING — Do not approve Gate 2</x:v>
       </x:c>
       <x:c r="B17" s="16"/>
       <x:c r="C17" s="16"/>
@@ -3848,7 +3957,7 @@
     </x:row>
     <x:row r="3" ht="18" hidden="0" customHeight="1">
       <x:c r="A3" s="3" t="str">
-        <x:v>BUS 331 Investments  |  Endicott College  |  Apply the approved Phase 1 Bear Case to the Phase 2 Portfolio</x:v>
+        <x:v>BUS 331 Investments | Stage 1: submit baseline; Stage 2: run the instructor-issued Scenario Reveal and remediation test</x:v>
       </x:c>
       <x:c r="B3" s="3"/>
       <x:c r="C3" s="3"/>
@@ -3864,33 +3973,39 @@
     <x:row r="4" ht="6" hidden="0" customHeight="1"/>
     <x:row r="5" ht="21.75" hidden="0" customHeight="1">
       <x:c r="B5" s="17" t="s">
-        <x:v>40</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C5" s="18"/>
       <x:c r="D5" s="17" t="s">
-        <x:v>41</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="E5" s="19" t="n">
         <x:v>500000</x:v>
       </x:c>
       <x:c r="F5" s="20" t="s">
-        <x:v>42</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G5" s="21"/>
       <x:c r="H5" s="17" t="s">
-        <x:v>43</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="I5" s="22" t="str">
         <x:v>(from Phase 1)</x:v>
       </x:c>
       <x:c r="J5" s="23" t="s">
-        <x:v>44</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="6" hidden="0" customHeight="1"/>
+        <x:v>18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="6" hidden="0" customHeight="1">
+      <x:c r="H6" s="99" t="str">
+        <x:v>Scenario Release Packet ID:</x:v>
+      </x:c>
+      <x:c r="I6" s="99" t="str"/>
+      <x:c r="J6" s="99"/>
+    </x:row>
     <x:row r="7" ht="19.5" hidden="0" customHeight="1">
-      <x:c r="A7" s="4" t="s">
-        <x:v>45</x:v>
+      <x:c r="A7" s="4" t="str">
+        <x:v>  SECTION 1 — SCENARIO REVEAL ASSUMPTIONS  (enter only after instructor release)</x:v>
       </x:c>
       <x:c r="B7" s="4"/>
       <x:c r="C7" s="4"/>
@@ -3904,8 +4019,8 @@
       <x:c r="K7" s="4"/>
     </x:row>
     <x:row r="8" ht="31.5" hidden="0" customHeight="1">
-      <x:c r="A8" s="24" t="s">
-        <x:v>46</x:v>
+      <x:c r="A8" s="24" t="str">
+        <x:v>Stage 1: submit the baseline portfolio snapshot using your approved Phase 1 bear-case inputs. Stage 2: after the instructor issues a Scenario Reveal packet, copy the released inputs below exactly. These values drive the remediation test; do not soften them, change the client mandate, or enter values before the release.</x:v>
       </x:c>
       <x:c r="B8" s="24"/>
       <x:c r="C8" s="24"/>
@@ -3919,17 +4034,19 @@
       <x:c r="K8" s="24"/>
     </x:row>
     <x:row r="9" ht="30" hidden="0" customHeight="1">
-      <x:c r="B9" s="25" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="C9" s="25" t="s">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="D9" s="25" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="E9" s="26" t="s">
-        <x:v>50</x:v>
+      <x:c r="B9" s="25" t="str">
+        <x:v>Asset Class</x:v>
+      </x:c>
+      <x:c r="C9" s="25" t="str">
+        <x:v>Scenario Reveal
+E(R) Input</x:v>
+      </x:c>
+      <x:c r="D9" s="25" t="str">
+        <x:v>Scenario Reveal
+Std Dev (σ)</x:v>
+      </x:c>
+      <x:c r="E9" s="26" t="str">
+        <x:v>Instructor packet / source reference</x:v>
       </x:c>
       <x:c r="F9" s="26"/>
       <x:c r="G9" s="26"/>
@@ -3940,7 +4057,7 @@
     </x:row>
     <x:row r="10" ht="21.75" hidden="0" customHeight="1">
       <x:c r="B10" s="27" t="s">
-        <x:v>51</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="C10" s="21"/>
       <x:c r="D10" s="21"/>
@@ -3954,7 +4071,7 @@
     </x:row>
     <x:row r="11" ht="21.75" hidden="0" customHeight="1">
       <x:c r="B11" s="29" t="s">
-        <x:v>52</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C11" s="21"/>
       <x:c r="D11" s="21"/>
@@ -3968,7 +4085,7 @@
     </x:row>
     <x:row r="12" ht="21.75" hidden="0" customHeight="1">
       <x:c r="B12" s="27" t="s">
-        <x:v>53</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C12" s="21"/>
       <x:c r="D12" s="21"/>
@@ -3983,7 +4100,7 @@
     <x:row r="13" ht="7.5" hidden="0" customHeight="1"/>
     <x:row r="14" ht="19.5" hidden="0" customHeight="1">
       <x:c r="A14" s="4" t="str">
-        <x:v>  SECTION 2 — BASE CASE PORTFOLIO  (enter Phase 2 Workstream A weights)</x:v>
+        <x:v>  SECTION 2 — BASELINE PORTFOLIO  (submitted before Scenario Reveal)</x:v>
       </x:c>
       <x:c r="B14" s="4"/>
       <x:c r="C14" s="4"/>
@@ -3998,7 +4115,7 @@
     </x:row>
     <x:row r="15" ht="31.5" hidden="0" customHeight="1">
       <x:c r="A15" s="8" t="str">
-        <x:v>Enter the Solver-supported weights from Phase 2 Workstream A for this client. Weights must sum to 100%. The Base Case return and risk metrics auto-calculate.</x:v>
+        <x:v>Enter the Solver-supported baseline weights from Workstream A and submit the baseline snapshot before the Scenario Reveal. Keep that original evidence in Canvas. Do not overwrite the submitted allocation after the release; document all changes in Section 5.</x:v>
       </x:c>
       <x:c r="B15" s="8"/>
       <x:c r="C15" s="8"/>
@@ -4013,36 +4130,39 @@
     </x:row>
     <x:row r="16" ht="33.75" hidden="0" customHeight="1">
       <x:c r="B16" s="25" t="s">
-        <x:v>47</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C16" s="25" t="str">
         <x:v>Weight
 (Workstream A)</x:v>
       </x:c>
       <x:c r="D16" s="25" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="E16" s="25" t="s">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="F16" s="25" t="s">
-        <x:v>56</x:v>
-      </x:c>
-      <x:c r="G16" s="25" t="s">
-        <x:v>57</x:v>
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="E16" s="25" t="str">
+        <x:v>Baseline Case
+E(R) Contrib.</x:v>
+      </x:c>
+      <x:c r="F16" s="25" t="str">
+        <x:v>Scenario Reveal
+Return Contrib.</x:v>
+      </x:c>
+      <x:c r="G16" s="25" t="str">
+        <x:v>Scenario Reveal
+$ P&amp;L</x:v>
       </x:c>
       <x:c r="H16" s="25" t="s">
-        <x:v>58</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="I16" s="30" t="s">
-        <x:v>59</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="J16" s="30"/>
       <x:c r="K16" s="30"/>
     </x:row>
     <x:row r="17" ht="21.75" hidden="0" customHeight="1">
       <x:c r="B17" s="27" t="s">
-        <x:v>51</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="C17" s="21"/>
       <x:c r="D17" s="31" t="str">
@@ -4062,7 +4182,7 @@
     </x:row>
     <x:row r="18" ht="21.75" hidden="0" customHeight="1">
       <x:c r="B18" s="29" t="s">
-        <x:v>52</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C18" s="21"/>
       <x:c r="D18" s="31" t="str">
@@ -4082,7 +4202,7 @@
     </x:row>
     <x:row r="19" ht="21.75" hidden="0" customHeight="1">
       <x:c r="B19" s="27" t="s">
-        <x:v>53</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C19" s="21"/>
       <x:c r="D19" s="31" t="str">
@@ -4102,7 +4222,7 @@
     </x:row>
     <x:row r="20" ht="24" hidden="0" customHeight="1">
       <x:c r="A20" s="38" t="s">
-        <x:v>60</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="B20" s="38"/>
       <x:c r="C20" s="39" t="n">
@@ -4125,8 +4245,8 @@
         <x:f aca="0">IFERROR(SUM(G17:G19),"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H20" s="40" t="s">
-        <x:v>61</x:v>
+      <x:c r="H20" s="40" t="str">
+        <x:v>← Scenario Reveal return must be ≥ IPS Tripwire (cell G5). See Section 4 verdict below.</x:v>
       </x:c>
       <x:c r="I20" s="40"/>
       <x:c r="J20" s="40"/>
@@ -4134,8 +4254,8 @@
     </x:row>
     <x:row r="21" ht="7.5" hidden="0" customHeight="1"/>
     <x:row r="22" ht="19.5" hidden="0" customHeight="1">
-      <x:c r="A22" s="4" t="s">
-        <x:v>62</x:v>
+      <x:c r="A22" s="4" t="str">
+        <x:v>  SECTION 3 — RISK METRICS  (Baseline &amp; Scenario Reveal)</x:v>
       </x:c>
       <x:c r="B22" s="4"/>
       <x:c r="C22" s="4"/>
@@ -4150,7 +4270,7 @@
     </x:row>
     <x:row r="23" ht="31.5" hidden="0" customHeight="1">
       <x:c r="A23" s="8" t="str">
-        <x:v>Enter portfolio risk metrics for BOTH the Base Case and Bear Case. Beta and σ come from the Phase 2 allocation and selected holdings. Sharpe Ratio is calculated automatically using the formula below.</x:v>
+        <x:v>Enter portfolio risk metrics for the submitted baseline and the Scenario Reveal. Beta and σ come from the Phase 2 allocation and selected holdings. Sharpe Ratio calculates automatically using the formula below.</x:v>
       </x:c>
       <x:c r="B23" s="8"/>
       <x:c r="C23" s="8"/>
@@ -4165,20 +4285,20 @@
     </x:row>
     <x:row r="24" ht="30" hidden="0" customHeight="1">
       <x:c r="B24" s="25" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C24" s="25" t="str">
+        <x:v>Baseline
+(Phase 2)</x:v>
+      </x:c>
+      <x:c r="D24" s="25" t="str">
+        <x:v>Scenario Reveal</x:v>
+      </x:c>
+      <x:c r="E24" s="25" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="F24" s="26" t="s">
         <x:v>28</x:v>
-      </x:c>
-      <x:c r="C24" s="25" t="str">
-        <x:v>Base Case
-(Phase 2)</x:v>
-      </x:c>
-      <x:c r="D24" s="25" t="s">
-        <x:v>63</x:v>
-      </x:c>
-      <x:c r="E24" s="25" t="s">
-        <x:v>64</x:v>
-      </x:c>
-      <x:c r="F24" s="26" t="s">
-        <x:v>65</x:v>
       </x:c>
       <x:c r="G24" s="26"/>
       <x:c r="H24" s="26"/>
@@ -4188,11 +4308,11 @@
     </x:row>
     <x:row r="25" ht="21.75" hidden="0" customHeight="1">
       <x:c r="B25" s="17" t="s">
-        <x:v>66</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="C25" s="21"/>
       <x:c r="D25" s="40" t="s">
-        <x:v>67</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E25" s="40"/>
       <x:c r="F25" s="40"/>
@@ -4204,7 +4324,7 @@
     </x:row>
     <x:row r="26" ht="25.5" hidden="0" customHeight="1">
       <x:c r="B26" s="10" t="s">
-        <x:v>36</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C26" s="41"/>
       <x:c r="D26" s="42"/>
@@ -4212,7 +4332,7 @@
         <x:v>From Phase 2 security selection — weighted average beta of all holdings</x:v>
       </x:c>
       <x:c r="F26" s="44" t="s">
-        <x:v>68</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="G26" s="44"/>
       <x:c r="H26" s="44"/>
@@ -4222,7 +4342,7 @@
     </x:row>
     <x:row r="27" ht="25.5" hidden="0" customHeight="1">
       <x:c r="B27" s="12" t="s">
-        <x:v>69</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="C27" s="21"/>
       <x:c r="D27" s="21"/>
@@ -4230,7 +4350,7 @@
         <x:v>From Phase 2 CME Matrix — portfolio σ from Solver output</x:v>
       </x:c>
       <x:c r="F27" s="44" t="s">
-        <x:v>70</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="G27" s="44"/>
       <x:c r="H27" s="44"/>
@@ -4240,7 +4360,7 @@
     </x:row>
     <x:row r="28" ht="25.5" hidden="0" customHeight="1">
       <x:c r="B28" s="10" t="s">
-        <x:v>71</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="C28" s="41" t="str">
         <x:f aca="0">IFERROR((E20-$C$25)/C27,"")</x:f>
@@ -4249,10 +4369,10 @@
         <x:f aca="0">IFERROR((F20-$C$25)/D27,"")</x:f>
       </x:c>
       <x:c r="E28" s="43" t="s">
-        <x:v>72</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="F28" s="44" t="s">
-        <x:v>73</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="G28" s="44"/>
       <x:c r="H28" s="44"/>
@@ -4261,21 +4381,21 @@
       <x:c r="K28" s="44"/>
     </x:row>
     <x:row r="29" ht="25.5" hidden="0" customHeight="1">
-      <x:c r="B29" s="12" t="s">
-        <x:v>74</x:v>
+      <x:c r="B29" s="12" t="str">
+        <x:v>Max Drawdown (Scenario Reveal)</x:v>
       </x:c>
       <x:c r="C29" s="45" t="s">
-        <x:v>75</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="D29" s="32" t="n">
         <x:f aca="0">IFERROR(F20,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E29" s="43" t="s">
-        <x:v>76</x:v>
-      </x:c>
-      <x:c r="F29" s="44" t="s">
-        <x:v>77</x:v>
+      <x:c r="E29" s="43" t="str">
+        <x:v>Total Scenario Reveal Return (Section 2 row 20)</x:v>
+      </x:c>
+      <x:c r="F29" s="44" t="str">
+        <x:v>Must be ≥ IPS Tripwire (cell G5). This drives the Scenario Reveal verdict.</x:v>
       </x:c>
       <x:c r="G29" s="44"/>
       <x:c r="H29" s="44"/>
@@ -4285,15 +4405,15 @@
     </x:row>
     <x:row r="30" ht="25.5" hidden="0" customHeight="1">
       <x:c r="B30" s="10" t="s">
-        <x:v>78</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="C30" s="42"/>
       <x:c r="D30" s="42"/>
       <x:c r="E30" s="43" t="s">
-        <x:v>79</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="F30" s="44" t="s">
-        <x:v>80</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="G30" s="44"/>
       <x:c r="H30" s="44"/>
@@ -4303,8 +4423,8 @@
     </x:row>
     <x:row r="31" ht="7.5" hidden="0" customHeight="1"/>
     <x:row r="32" ht="19.5" hidden="0" customHeight="1">
-      <x:c r="A32" s="4" t="s">
-        <x:v>81</x:v>
+      <x:c r="A32" s="4" t="str">
+        <x:v>  SECTION 4 — SCENARIO REVEAL VERDICT</x:v>
       </x:c>
       <x:c r="B32" s="4"/>
       <x:c r="C32" s="4"/>
@@ -4319,19 +4439,19 @@
     </x:row>
     <x:row r="33" ht="30" hidden="0" customHeight="1">
       <x:c r="B33" s="25" t="s">
-        <x:v>82</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="C33" s="25" t="s">
-        <x:v>83</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="D33" s="25" t="s">
-        <x:v>84</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="E33" s="25" t="s">
-        <x:v>85</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="F33" s="26" t="s">
-        <x:v>86</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="G33" s="26"/>
       <x:c r="H33" s="26"/>
@@ -4341,7 +4461,7 @@
     </x:row>
     <x:row r="34" ht="25.5" hidden="0" customHeight="1">
       <x:c r="B34" s="10" t="s">
-        <x:v>87</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="C34" s="32" t="n">
         <x:f aca="0">$G$5</x:f>
@@ -4359,7 +4479,7 @@
         <x:f aca="0">IF(D34="","",IF(D34&gt;=C34,"✓ PASS","✗ FAIL — RE-ALLOCATE"))</x:f>
       </x:c>
       <x:c r="G34" s="47" t="str">
-        <x:f aca="0">IF(D34="","",IF(D34&gt;=C34,"Portfolio passes IPS mandate. No re-allocation required. Proceed to Section 6 (Final Metrics).","FAIL: Portfolio breaches IPS Tripwire by "&amp;TEXT(ABS(D34-C34),"0.0%")&amp;". Complete Section 5 (Re-allocation) to bring portfolio within mandate before submitting."))</x:f>
+        <x:f aca="0">IF(D34="","",IF(D34&gt;=C34,"Scenario Reveal shows PASS. Stop and report this result to the instructor; do not use a PASS to skip the remediation checkpoint.","BREACH: Portfolio misses the IPS Tripwire by "&amp;TEXT(ABS(D34-C34),"0.0%")&amp;". Complete Section 5 with a real trade, trade-off, and full re-test before Gate 2."))</x:f>
       </x:c>
       <x:c r="H34" s="47"/>
       <x:c r="I34" s="47"/>
@@ -4368,7 +4488,7 @@
     </x:row>
     <x:row r="35" ht="25.5" hidden="0" customHeight="1">
       <x:c r="B35" s="12" t="s">
-        <x:v>88</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C35" s="21"/>
       <x:c r="D35" s="32" t="str">
@@ -4382,17 +4502,21 @@
         <x:f aca="0">IF(D35="","",IF(D35&lt;=C35,"✓ PASS","✗ EXCEED"))</x:f>
       </x:c>
       <x:c r="G35" s="48" t="s">
-        <x:v>89</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="H35" s="48"/>
       <x:c r="I35" s="48"/>
       <x:c r="J35" s="48"/>
       <x:c r="K35" s="48"/>
     </x:row>
-    <x:row r="36" ht="7.5" hidden="0" customHeight="1"/>
+    <x:row r="36" ht="7.5" hidden="0" customHeight="1">
+      <x:c r="A36" t="str">
+        <x:v>  SECTION 5 — REQUIRED REMEDIATION &amp; RE-TEST</x:v>
+      </x:c>
+    </x:row>
     <x:row r="37" ht="19.5" hidden="0" customHeight="1">
-      <x:c r="A37" s="49" t="s">
-        <x:v>90</x:v>
+      <x:c r="A37" s="49" t="str">
+        <x:v>  A breach requires a real portfolio change, stated trade-off, and full re-test</x:v>
       </x:c>
       <x:c r="B37" s="49"/>
       <x:c r="C37" s="49"/>
@@ -4406,8 +4530,8 @@
       <x:c r="K37" s="49"/>
     </x:row>
     <x:row r="38" ht="31.5" hidden="0" customHeight="1">
-      <x:c r="A38" s="50" t="s">
-        <x:v>91</x:v>
+      <x:c r="A38" s="50" t="str">
+        <x:v>The Scenario Reveal is calibrated to test a client condition the baseline may not absorb. Document what was sold or reduced, what was bought or increased, old and new weights, dollar impact, rationale, and the trade-off. If the result is unexpectedly PASS, stop and report it to the instructor; do not skip the checkpoint.</x:v>
       </x:c>
       <x:c r="B38" s="50"/>
       <x:c r="C38" s="50"/>
@@ -4422,7 +4546,7 @@
     </x:row>
     <x:row r="39" ht="18" hidden="0" customHeight="1">
       <x:c r="A39" s="51" t="s">
-        <x:v>92</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="B39" s="51"/>
       <x:c r="C39" s="51"/>
@@ -4437,22 +4561,22 @@
     </x:row>
     <x:row r="40" ht="30" hidden="0" customHeight="1">
       <x:c r="B40" s="25" t="s">
-        <x:v>93</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C40" s="25" t="s">
-        <x:v>94</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="D40" s="25" t="s">
-        <x:v>95</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="E40" s="25" t="s">
-        <x:v>96</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="F40" s="25" t="s">
-        <x:v>97</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="G40" s="26" t="s">
-        <x:v>98</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="H40" s="26"/>
       <x:c r="I40" s="26"/>
@@ -4545,7 +4669,7 @@
     </x:row>
     <x:row r="47" ht="21.75" hidden="0" customHeight="1">
       <x:c r="A47" s="52" t="s">
-        <x:v>99</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="B47" s="52"/>
       <x:c r="C47" s="52"/>
@@ -4554,7 +4678,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E47" s="40" t="s">
-        <x:v>100</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="F47" s="40"/>
       <x:c r="G47" s="40"/>
@@ -4565,8 +4689,8 @@
     </x:row>
     <x:row r="48" ht="7.5" hidden="0" customHeight="1"/>
     <x:row r="49" ht="18" hidden="0" customHeight="1">
-      <x:c r="A49" s="51" t="s">
-        <x:v>101</x:v>
+      <x:c r="A49" s="51" t="str">
+        <x:v>  Part B — Revised Scenario Reveal Result  (confirm the corrective portfolio now passes)</x:v>
       </x:c>
       <x:c r="B49" s="51"/>
       <x:c r="C49" s="51"/>
@@ -4580,8 +4704,8 @@
       <x:c r="K49" s="51"/>
     </x:row>
     <x:row r="50" ht="31.5" hidden="0" customHeight="1">
-      <x:c r="A50" s="8" t="s">
-        <x:v>102</x:v>
+      <x:c r="A50" s="8" t="str">
+        <x:v>Using the new weights from Part A, recalculate the released scenario result. The result must be at or above the IPS Tripwire. Show the calculation clearly and retain the baseline evidence separately.</x:v>
       </x:c>
       <x:c r="B50" s="8"/>
       <x:c r="C50" s="8"/>
@@ -4596,22 +4720,22 @@
     </x:row>
     <x:row r="51" ht="30" hidden="0" customHeight="1">
       <x:c r="B51" s="25" t="s">
-        <x:v>47</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C51" s="25" t="s">
-        <x:v>103</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="D51" s="25" t="s">
-        <x:v>104</x:v>
-      </x:c>
-      <x:c r="E51" s="25" t="s">
-        <x:v>105</x:v>
-      </x:c>
-      <x:c r="F51" s="25" t="s">
-        <x:v>106</x:v>
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="E51" s="25" t="str">
+        <x:v>Scenario Reveal E(R)</x:v>
+      </x:c>
+      <x:c r="F51" s="25" t="str">
+        <x:v>Wtd Scenario Contribution</x:v>
       </x:c>
       <x:c r="G51" s="26" t="s">
-        <x:v>107</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="H51" s="26"/>
       <x:c r="I51" s="26"/>
@@ -4620,7 +4744,7 @@
     </x:row>
     <x:row r="52" ht="21.75" hidden="0" customHeight="1">
       <x:c r="B52" s="27" t="s">
-        <x:v>51</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="C52" s="21"/>
       <x:c r="D52" s="31" t="str">
@@ -4643,7 +4767,7 @@
     </x:row>
     <x:row r="53" ht="21.75" hidden="0" customHeight="1">
       <x:c r="B53" s="29" t="s">
-        <x:v>52</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C53" s="21"/>
       <x:c r="D53" s="31" t="str">
@@ -4666,7 +4790,7 @@
     </x:row>
     <x:row r="54" ht="21.75" hidden="0" customHeight="1">
       <x:c r="B54" s="27" t="s">
-        <x:v>53</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C54" s="21"/>
       <x:c r="D54" s="31" t="str">
@@ -4689,7 +4813,7 @@
     </x:row>
     <x:row r="55" ht="24" hidden="0" customHeight="1">
       <x:c r="A55" s="38" t="s">
-        <x:v>108</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="B55" s="38"/>
       <x:c r="C55" s="32" t="n">
@@ -4712,7 +4836,7 @@
     </x:row>
     <x:row r="56" ht="25.5" hidden="0" customHeight="1">
       <x:c r="B56" s="10" t="s">
-        <x:v>109</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C56" s="32" t="n">
         <x:f aca="0">$G$5</x:f>
@@ -4729,8 +4853,8 @@
       <x:c r="F56" s="46" t="str">
         <x:f aca="0">IF(D56="","",IF(D56&gt;=$G$5,"✓ REVISED PASS","✗ STILL FAILING — ADJUST FURTHER"))</x:f>
       </x:c>
-      <x:c r="G56" s="48" t="s">
-        <x:v>110</x:v>
+      <x:c r="G56" s="48" t="str">
+        <x:v>Revised Scenario Reveal return must be ≥ IPS Tripwire (G5). If still failing, make a further documented adjustment and re-test.</x:v>
       </x:c>
       <x:c r="H56" s="48"/>
       <x:c r="I56" s="48"/>
@@ -4739,8 +4863,8 @@
     </x:row>
     <x:row r="57" ht="7.5" hidden="0" customHeight="1"/>
     <x:row r="58" ht="19.5" hidden="0" customHeight="1">
-      <x:c r="A58" s="4" t="s">
-        <x:v>111</x:v>
+      <x:c r="A58" s="4" t="str">
+        <x:v>  SECTION 6 — FINAL RISK METRICS SUMMARY  (for Gate 2 submission)</x:v>
       </x:c>
       <x:c r="B58" s="4"/>
       <x:c r="C58" s="4"/>
@@ -4755,7 +4879,7 @@
     </x:row>
     <x:row r="59" ht="31.5" hidden="0" customHeight="1">
       <x:c r="A59" s="8" t="str">
-        <x:v>These are the final numbers your team submits. If you re-allocated in Section 5, use the revised portfolio metrics here. If the original portfolio passed, carry forward the verified Phase 2 metrics.</x:v>
+        <x:v>These are the final Gate 2 numbers. Use the revised portfolio metrics after the Scenario Reveal remediation and retain the pre-reveal baseline snapshot as a separate submitted record.</x:v>
       </x:c>
       <x:c r="B59" s="8"/>
       <x:c r="C59" s="8"/>
@@ -4770,16 +4894,16 @@
     </x:row>
     <x:row r="60" ht="30" hidden="0" customHeight="1">
       <x:c r="B60" s="25" t="s">
-        <x:v>28</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C60" s="25" t="s">
-        <x:v>112</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="D60" s="25" t="s">
-        <x:v>113</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="E60" s="26" t="s">
-        <x:v>114</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="F60" s="26"/>
       <x:c r="G60" s="26"/>
@@ -4790,11 +4914,11 @@
     </x:row>
     <x:row r="61" ht="24" hidden="0" customHeight="1">
       <x:c r="B61" s="10" t="s">
-        <x:v>36</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C61" s="42"/>
       <x:c r="D61" s="55" t="s">
-        <x:v>115</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="E61" s="44" t="str">
         <x:v>Weighted average β from the Phase 2 security-selection record</x:v>
@@ -4808,7 +4932,7 @@
     </x:row>
     <x:row r="62" ht="24" hidden="0" customHeight="1">
       <x:c r="B62" s="12" t="s">
-        <x:v>69</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="C62" s="21"/>
       <x:c r="D62" s="55" t="str">
@@ -4826,14 +4950,14 @@
     </x:row>
     <x:row r="63" ht="24" hidden="0" customHeight="1">
       <x:c r="B63" s="10" t="s">
-        <x:v>116</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C63" s="42"/>
       <x:c r="D63" s="55" t="s">
-        <x:v>117</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="E63" s="44" t="s">
-        <x:v>118</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F63" s="44"/>
       <x:c r="G63" s="44"/>
@@ -4843,15 +4967,15 @@
       <x:c r="K63" s="44"/>
     </x:row>
     <x:row r="64" ht="24" hidden="0" customHeight="1">
-      <x:c r="B64" s="12" t="s">
-        <x:v>33</x:v>
+      <x:c r="B64" s="12" t="str">
+        <x:v>Scenario Reveal Portfolio Return</x:v>
       </x:c>
       <x:c r="C64" s="21"/>
       <x:c r="D64" s="55" t="s">
-        <x:v>119</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="E64" s="44" t="s">
-        <x:v>120</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="F64" s="44"/>
       <x:c r="G64" s="44"/>
@@ -4861,15 +4985,15 @@
       <x:c r="K64" s="44"/>
     </x:row>
     <x:row r="65" ht="24" hidden="0" customHeight="1">
-      <x:c r="B65" s="10" t="s">
-        <x:v>121</x:v>
+      <x:c r="B65" s="10" t="str">
+        <x:v>Scenario Reveal $ P&amp;L</x:v>
       </x:c>
       <x:c r="C65" s="56"/>
       <x:c r="D65" s="55" t="s">
-        <x:v>122</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="E65" s="44" t="s">
-        <x:v>120</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="F65" s="44"/>
       <x:c r="G65" s="44"/>
@@ -4879,15 +5003,15 @@
       <x:c r="K65" s="44"/>
     </x:row>
     <x:row r="66" ht="24" hidden="0" customHeight="1">
-      <x:c r="B66" s="12" t="s">
-        <x:v>123</x:v>
+      <x:c r="B66" s="12" t="str">
+        <x:v>IPS Mandate Status after re-test</x:v>
       </x:c>
       <x:c r="C66" s="57"/>
       <x:c r="D66" s="55" t="s">
-        <x:v>124</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="E66" s="44" t="s">
-        <x:v>125</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="F66" s="44"/>
       <x:c r="G66" s="44"/>
@@ -4899,7 +5023,7 @@
     <x:row r="68" ht="7.5" hidden="0" customHeight="1"/>
     <x:row r="69" ht="19.5" hidden="0" customHeight="1">
       <x:c r="A69" s="4" t="s">
-        <x:v>126</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="B69" s="4"/>
       <x:c r="C69" s="4"/>
@@ -4914,10 +5038,10 @@
     </x:row>
     <x:row r="70" ht="18" hidden="0" customHeight="1">
       <x:c r="B70" s="58" t="s">
-        <x:v>127</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C70" s="7" t="s">
-        <x:v>128</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="D70" s="7"/>
       <x:c r="E70" s="7"/>
@@ -4930,10 +5054,10 @@
     </x:row>
     <x:row r="71" ht="18" hidden="0" customHeight="1">
       <x:c r="B71" s="59" t="s">
-        <x:v>127</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C71" s="7" t="s">
-        <x:v>129</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="D71" s="7"/>
       <x:c r="E71" s="7"/>
@@ -4946,10 +5070,10 @@
     </x:row>
     <x:row r="72" ht="18" hidden="0" customHeight="1">
       <x:c r="B72" s="60" t="s">
-        <x:v>127</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C72" s="7" t="s">
-        <x:v>130</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="D72" s="7"/>
       <x:c r="E72" s="7"/>
@@ -4962,10 +5086,10 @@
     </x:row>
     <x:row r="73" ht="18" hidden="0" customHeight="1">
       <x:c r="B73" s="61" t="s">
-        <x:v>127</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C73" s="7" t="s">
-        <x:v>131</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="D73" s="7"/>
       <x:c r="E73" s="7"/>
@@ -4978,10 +5102,10 @@
     </x:row>
     <x:row r="74" ht="18" hidden="0" customHeight="1">
       <x:c r="B74" s="62" t="s">
-        <x:v>127</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C74" s="7" t="s">
-        <x:v>132</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="D74" s="7"/>
       <x:c r="E74" s="7"/>
@@ -4994,10 +5118,10 @@
     </x:row>
     <x:row r="75" ht="18" hidden="0" customHeight="1">
       <x:c r="B75" s="63" t="s">
-        <x:v>127</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C75" s="7" t="s">
-        <x:v>133</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="D75" s="7"/>
       <x:c r="E75" s="7"/>
@@ -5075,6 +5199,7 @@
     <x:mergeCell ref="C73:K73"/>
     <x:mergeCell ref="C74:K74"/>
     <x:mergeCell ref="C75:K75"/>
+    <x:mergeCell ref="I6:J6"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="C20:C20">
     <x:cfRule type="cellIs" dxfId="0" priority="2" aboveAverage="0" percent="0" bottom="0" operator="equal" rank="0" equalAverage="0">
@@ -5123,7 +5248,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0e5bfc99836542cb"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re076e6bd48fe45d0"/>
 </x:worksheet>
 </file>
 
@@ -5161,7 +5286,7 @@
     </x:row>
     <x:row r="3" ht="18" hidden="0" customHeight="1">
       <x:c r="A3" s="3" t="str">
-        <x:v>BUS 331 Investments  |  Endicott College  |  Apply the approved Phase 1 Bear Case to the Phase 2 Portfolio</x:v>
+        <x:v>BUS 331 Investments | Stage 1: submit baseline; Stage 2: run the instructor-issued Scenario Reveal and remediation test</x:v>
       </x:c>
       <x:c r="B3" s="3"/>
       <x:c r="C3" s="3"/>
@@ -5177,33 +5302,39 @@
     <x:row r="4" ht="6" hidden="0" customHeight="1"/>
     <x:row r="5" ht="21.75" hidden="0" customHeight="1">
       <x:c r="B5" s="17" t="s">
-        <x:v>40</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C5" s="18"/>
       <x:c r="D5" s="17" t="s">
-        <x:v>41</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="E5" s="19" t="n">
         <x:v>500000</x:v>
       </x:c>
       <x:c r="F5" s="20" t="s">
-        <x:v>42</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G5" s="21"/>
       <x:c r="H5" s="17" t="s">
-        <x:v>43</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="I5" s="22" t="str">
         <x:v>(from Phase 1)</x:v>
       </x:c>
       <x:c r="J5" s="23" t="s">
-        <x:v>44</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="6" hidden="0" customHeight="1"/>
+        <x:v>18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="6" hidden="0" customHeight="1">
+      <x:c r="H6" s="99" t="str">
+        <x:v>Scenario Release Packet ID:</x:v>
+      </x:c>
+      <x:c r="I6" s="99" t="str"/>
+      <x:c r="J6" s="99"/>
+    </x:row>
     <x:row r="7" ht="19.5" hidden="0" customHeight="1">
-      <x:c r="A7" s="4" t="s">
-        <x:v>45</x:v>
+      <x:c r="A7" s="4" t="str">
+        <x:v>  SECTION 1 — SCENARIO REVEAL ASSUMPTIONS  (enter only after instructor release)</x:v>
       </x:c>
       <x:c r="B7" s="4"/>
       <x:c r="C7" s="4"/>
@@ -5217,8 +5348,8 @@
       <x:c r="K7" s="4"/>
     </x:row>
     <x:row r="8" ht="31.5" hidden="0" customHeight="1">
-      <x:c r="A8" s="24" t="s">
-        <x:v>46</x:v>
+      <x:c r="A8" s="24" t="str">
+        <x:v>Stage 1: submit the baseline portfolio snapshot using your approved Phase 1 bear-case inputs. Stage 2: after the instructor issues a Scenario Reveal packet, copy the released inputs below exactly. These values drive the remediation test; do not soften them, change the client mandate, or enter values before the release.</x:v>
       </x:c>
       <x:c r="B8" s="24"/>
       <x:c r="C8" s="24"/>
@@ -5232,17 +5363,19 @@
       <x:c r="K8" s="24"/>
     </x:row>
     <x:row r="9" ht="30" hidden="0" customHeight="1">
-      <x:c r="B9" s="25" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="C9" s="25" t="s">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="D9" s="25" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="E9" s="26" t="s">
-        <x:v>50</x:v>
+      <x:c r="B9" s="25" t="str">
+        <x:v>Asset Class</x:v>
+      </x:c>
+      <x:c r="C9" s="25" t="str">
+        <x:v>Scenario Reveal
+E(R) Input</x:v>
+      </x:c>
+      <x:c r="D9" s="25" t="str">
+        <x:v>Scenario Reveal
+Std Dev (σ)</x:v>
+      </x:c>
+      <x:c r="E9" s="26" t="str">
+        <x:v>Instructor packet / source reference</x:v>
       </x:c>
       <x:c r="F9" s="26"/>
       <x:c r="G9" s="26"/>
@@ -5253,7 +5386,7 @@
     </x:row>
     <x:row r="10" ht="21.75" hidden="0" customHeight="1">
       <x:c r="B10" s="27" t="s">
-        <x:v>51</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="C10" s="21"/>
       <x:c r="D10" s="21"/>
@@ -5267,7 +5400,7 @@
     </x:row>
     <x:row r="11" ht="21.75" hidden="0" customHeight="1">
       <x:c r="B11" s="29" t="s">
-        <x:v>52</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C11" s="21"/>
       <x:c r="D11" s="21"/>
@@ -5281,7 +5414,7 @@
     </x:row>
     <x:row r="12" ht="21.75" hidden="0" customHeight="1">
       <x:c r="B12" s="27" t="s">
-        <x:v>53</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C12" s="21"/>
       <x:c r="D12" s="21"/>
@@ -5296,7 +5429,7 @@
     <x:row r="13" ht="7.5" hidden="0" customHeight="1"/>
     <x:row r="14" ht="19.5" hidden="0" customHeight="1">
       <x:c r="A14" s="4" t="str">
-        <x:v>  SECTION 2 — BASE CASE PORTFOLIO  (enter Phase 2 Workstream A weights)</x:v>
+        <x:v>  SECTION 2 — BASELINE PORTFOLIO  (submitted before Scenario Reveal)</x:v>
       </x:c>
       <x:c r="B14" s="4"/>
       <x:c r="C14" s="4"/>
@@ -5311,7 +5444,7 @@
     </x:row>
     <x:row r="15" ht="31.5" hidden="0" customHeight="1">
       <x:c r="A15" s="8" t="str">
-        <x:v>Enter the Solver-supported weights from Phase 2 Workstream A for this client. Weights must sum to 100%. The Base Case return and risk metrics auto-calculate.</x:v>
+        <x:v>Enter the Solver-supported baseline weights from Workstream A and submit the baseline snapshot before the Scenario Reveal. Keep that original evidence in Canvas. Do not overwrite the submitted allocation after the release; document all changes in Section 5.</x:v>
       </x:c>
       <x:c r="B15" s="8"/>
       <x:c r="C15" s="8"/>
@@ -5326,36 +5459,39 @@
     </x:row>
     <x:row r="16" ht="33.75" hidden="0" customHeight="1">
       <x:c r="B16" s="25" t="s">
-        <x:v>47</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C16" s="25" t="str">
         <x:v>Weight
 (Workstream A)</x:v>
       </x:c>
       <x:c r="D16" s="25" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="E16" s="25" t="s">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="F16" s="25" t="s">
-        <x:v>56</x:v>
-      </x:c>
-      <x:c r="G16" s="25" t="s">
-        <x:v>57</x:v>
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="E16" s="25" t="str">
+        <x:v>Baseline Case
+E(R) Contrib.</x:v>
+      </x:c>
+      <x:c r="F16" s="25" t="str">
+        <x:v>Scenario Reveal
+Return Contrib.</x:v>
+      </x:c>
+      <x:c r="G16" s="25" t="str">
+        <x:v>Scenario Reveal
+$ P&amp;L</x:v>
       </x:c>
       <x:c r="H16" s="25" t="s">
-        <x:v>58</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="I16" s="30" t="s">
-        <x:v>59</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="J16" s="30"/>
       <x:c r="K16" s="30"/>
     </x:row>
     <x:row r="17" ht="21.75" hidden="0" customHeight="1">
       <x:c r="B17" s="27" t="s">
-        <x:v>51</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="C17" s="21"/>
       <x:c r="D17" s="31" t="str">
@@ -5375,7 +5511,7 @@
     </x:row>
     <x:row r="18" ht="21.75" hidden="0" customHeight="1">
       <x:c r="B18" s="29" t="s">
-        <x:v>52</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C18" s="21"/>
       <x:c r="D18" s="31" t="str">
@@ -5395,7 +5531,7 @@
     </x:row>
     <x:row r="19" ht="21.75" hidden="0" customHeight="1">
       <x:c r="B19" s="27" t="s">
-        <x:v>53</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C19" s="21"/>
       <x:c r="D19" s="31" t="str">
@@ -5415,7 +5551,7 @@
     </x:row>
     <x:row r="20" ht="24" hidden="0" customHeight="1">
       <x:c r="A20" s="38" t="s">
-        <x:v>60</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="B20" s="38"/>
       <x:c r="C20" s="39" t="n">
@@ -5438,8 +5574,8 @@
         <x:f aca="0">IFERROR(SUM(G17:G19),"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H20" s="40" t="s">
-        <x:v>61</x:v>
+      <x:c r="H20" s="40" t="str">
+        <x:v>← Scenario Reveal return must be ≥ IPS Tripwire (cell G5). See Section 4 verdict below.</x:v>
       </x:c>
       <x:c r="I20" s="40"/>
       <x:c r="J20" s="40"/>
@@ -5447,8 +5583,8 @@
     </x:row>
     <x:row r="21" ht="7.5" hidden="0" customHeight="1"/>
     <x:row r="22" ht="19.5" hidden="0" customHeight="1">
-      <x:c r="A22" s="4" t="s">
-        <x:v>62</x:v>
+      <x:c r="A22" s="4" t="str">
+        <x:v>  SECTION 3 — RISK METRICS  (Baseline &amp; Scenario Reveal)</x:v>
       </x:c>
       <x:c r="B22" s="4"/>
       <x:c r="C22" s="4"/>
@@ -5463,7 +5599,7 @@
     </x:row>
     <x:row r="23" ht="31.5" hidden="0" customHeight="1">
       <x:c r="A23" s="8" t="str">
-        <x:v>Enter portfolio risk metrics for BOTH the Base Case and Bear Case. Beta and σ come from the Phase 2 allocation and selected holdings. Sharpe Ratio is calculated automatically using the formula below.</x:v>
+        <x:v>Enter portfolio risk metrics for the submitted baseline and the Scenario Reveal. Beta and σ come from the Phase 2 allocation and selected holdings. Sharpe Ratio calculates automatically using the formula below.</x:v>
       </x:c>
       <x:c r="B23" s="8"/>
       <x:c r="C23" s="8"/>
@@ -5478,20 +5614,20 @@
     </x:row>
     <x:row r="24" ht="30" hidden="0" customHeight="1">
       <x:c r="B24" s="25" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C24" s="25" t="str">
+        <x:v>Baseline
+(Phase 2)</x:v>
+      </x:c>
+      <x:c r="D24" s="25" t="str">
+        <x:v>Scenario Reveal</x:v>
+      </x:c>
+      <x:c r="E24" s="25" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="F24" s="26" t="s">
         <x:v>28</x:v>
-      </x:c>
-      <x:c r="C24" s="25" t="str">
-        <x:v>Base Case
-(Phase 2)</x:v>
-      </x:c>
-      <x:c r="D24" s="25" t="s">
-        <x:v>63</x:v>
-      </x:c>
-      <x:c r="E24" s="25" t="s">
-        <x:v>64</x:v>
-      </x:c>
-      <x:c r="F24" s="26" t="s">
-        <x:v>65</x:v>
       </x:c>
       <x:c r="G24" s="26"/>
       <x:c r="H24" s="26"/>
@@ -5501,11 +5637,11 @@
     </x:row>
     <x:row r="25" ht="21.75" hidden="0" customHeight="1">
       <x:c r="B25" s="17" t="s">
-        <x:v>66</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="C25" s="21"/>
       <x:c r="D25" s="40" t="s">
-        <x:v>67</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E25" s="40"/>
       <x:c r="F25" s="40"/>
@@ -5517,7 +5653,7 @@
     </x:row>
     <x:row r="26" ht="25.5" hidden="0" customHeight="1">
       <x:c r="B26" s="10" t="s">
-        <x:v>36</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C26" s="41"/>
       <x:c r="D26" s="42"/>
@@ -5525,7 +5661,7 @@
         <x:v>From Phase 2 security selection — weighted average beta of all holdings</x:v>
       </x:c>
       <x:c r="F26" s="44" t="s">
-        <x:v>68</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="G26" s="44"/>
       <x:c r="H26" s="44"/>
@@ -5535,7 +5671,7 @@
     </x:row>
     <x:row r="27" ht="25.5" hidden="0" customHeight="1">
       <x:c r="B27" s="12" t="s">
-        <x:v>69</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="C27" s="21"/>
       <x:c r="D27" s="21"/>
@@ -5543,7 +5679,7 @@
         <x:v>From Phase 2 CME Matrix — portfolio σ from Solver output</x:v>
       </x:c>
       <x:c r="F27" s="44" t="s">
-        <x:v>70</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="G27" s="44"/>
       <x:c r="H27" s="44"/>
@@ -5553,7 +5689,7 @@
     </x:row>
     <x:row r="28" ht="25.5" hidden="0" customHeight="1">
       <x:c r="B28" s="10" t="s">
-        <x:v>71</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="C28" s="41" t="str">
         <x:f aca="0">IFERROR((E20-$C$25)/C27,"")</x:f>
@@ -5562,10 +5698,10 @@
         <x:f aca="0">IFERROR((F20-$C$25)/D27,"")</x:f>
       </x:c>
       <x:c r="E28" s="43" t="s">
-        <x:v>72</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="F28" s="44" t="s">
-        <x:v>73</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="G28" s="44"/>
       <x:c r="H28" s="44"/>
@@ -5574,21 +5710,21 @@
       <x:c r="K28" s="44"/>
     </x:row>
     <x:row r="29" ht="25.5" hidden="0" customHeight="1">
-      <x:c r="B29" s="12" t="s">
-        <x:v>74</x:v>
+      <x:c r="B29" s="12" t="str">
+        <x:v>Max Drawdown (Scenario Reveal)</x:v>
       </x:c>
       <x:c r="C29" s="45" t="s">
-        <x:v>75</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="D29" s="32" t="n">
         <x:f aca="0">IFERROR(F20,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E29" s="43" t="s">
-        <x:v>76</x:v>
-      </x:c>
-      <x:c r="F29" s="44" t="s">
-        <x:v>77</x:v>
+      <x:c r="E29" s="43" t="str">
+        <x:v>Total Scenario Reveal Return (Section 2 row 20)</x:v>
+      </x:c>
+      <x:c r="F29" s="44" t="str">
+        <x:v>Must be ≥ IPS Tripwire (cell G5). This drives the Scenario Reveal verdict.</x:v>
       </x:c>
       <x:c r="G29" s="44"/>
       <x:c r="H29" s="44"/>
@@ -5598,15 +5734,15 @@
     </x:row>
     <x:row r="30" ht="25.5" hidden="0" customHeight="1">
       <x:c r="B30" s="10" t="s">
-        <x:v>78</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="C30" s="42"/>
       <x:c r="D30" s="42"/>
       <x:c r="E30" s="43" t="s">
-        <x:v>79</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="F30" s="44" t="s">
-        <x:v>80</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="G30" s="44"/>
       <x:c r="H30" s="44"/>
@@ -5616,8 +5752,8 @@
     </x:row>
     <x:row r="31" ht="7.5" hidden="0" customHeight="1"/>
     <x:row r="32" ht="19.5" hidden="0" customHeight="1">
-      <x:c r="A32" s="4" t="s">
-        <x:v>81</x:v>
+      <x:c r="A32" s="4" t="str">
+        <x:v>  SECTION 4 — SCENARIO REVEAL VERDICT</x:v>
       </x:c>
       <x:c r="B32" s="4"/>
       <x:c r="C32" s="4"/>
@@ -5632,19 +5768,19 @@
     </x:row>
     <x:row r="33" ht="30" hidden="0" customHeight="1">
       <x:c r="B33" s="25" t="s">
-        <x:v>82</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="C33" s="25" t="s">
-        <x:v>83</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="D33" s="25" t="s">
-        <x:v>84</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="E33" s="25" t="s">
-        <x:v>85</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="F33" s="26" t="s">
-        <x:v>86</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="G33" s="26"/>
       <x:c r="H33" s="26"/>
@@ -5654,7 +5790,7 @@
     </x:row>
     <x:row r="34" ht="25.5" hidden="0" customHeight="1">
       <x:c r="B34" s="10" t="s">
-        <x:v>87</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="C34" s="32" t="n">
         <x:f aca="0">$G$5</x:f>
@@ -5672,7 +5808,7 @@
         <x:f aca="0">IF(D34="","",IF(D34&gt;=C34,"✓ PASS","✗ FAIL — RE-ALLOCATE"))</x:f>
       </x:c>
       <x:c r="G34" s="47" t="str">
-        <x:f aca="0">IF(D34="","",IF(D34&gt;=C34,"Portfolio passes IPS mandate. No re-allocation required. Proceed to Section 6 (Final Metrics).","FAIL: Portfolio breaches IPS Tripwire by "&amp;TEXT(ABS(D34-C34),"0.0%")&amp;". Complete Section 5 (Re-allocation) to bring portfolio within mandate before submitting."))</x:f>
+        <x:f aca="0">IF(D34="","",IF(D34&gt;=C34,"Scenario Reveal shows PASS. Stop and report this result to the instructor; do not use a PASS to skip the remediation checkpoint.","BREACH: Portfolio misses the IPS Tripwire by "&amp;TEXT(ABS(D34-C34),"0.0%")&amp;". Complete Section 5 with a real trade, trade-off, and full re-test before Gate 2."))</x:f>
       </x:c>
       <x:c r="H34" s="47"/>
       <x:c r="I34" s="47"/>
@@ -5681,7 +5817,7 @@
     </x:row>
     <x:row r="35" ht="25.5" hidden="0" customHeight="1">
       <x:c r="B35" s="12" t="s">
-        <x:v>88</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C35" s="21"/>
       <x:c r="D35" s="32" t="str">
@@ -5695,17 +5831,21 @@
         <x:f aca="0">IF(D35="","",IF(D35&lt;=C35,"✓ PASS","✗ EXCEED"))</x:f>
       </x:c>
       <x:c r="G35" s="48" t="s">
-        <x:v>89</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="H35" s="48"/>
       <x:c r="I35" s="48"/>
       <x:c r="J35" s="48"/>
       <x:c r="K35" s="48"/>
     </x:row>
-    <x:row r="36" ht="7.5" hidden="0" customHeight="1"/>
+    <x:row r="36" ht="7.5" hidden="0" customHeight="1">
+      <x:c r="A36" t="str">
+        <x:v>  SECTION 5 — REQUIRED REMEDIATION &amp; RE-TEST</x:v>
+      </x:c>
+    </x:row>
     <x:row r="37" ht="19.5" hidden="0" customHeight="1">
-      <x:c r="A37" s="49" t="s">
-        <x:v>90</x:v>
+      <x:c r="A37" s="49" t="str">
+        <x:v>  A breach requires a real portfolio change, stated trade-off, and full re-test</x:v>
       </x:c>
       <x:c r="B37" s="49"/>
       <x:c r="C37" s="49"/>
@@ -5719,8 +5859,8 @@
       <x:c r="K37" s="49"/>
     </x:row>
     <x:row r="38" ht="31.5" hidden="0" customHeight="1">
-      <x:c r="A38" s="50" t="s">
-        <x:v>91</x:v>
+      <x:c r="A38" s="50" t="str">
+        <x:v>The Scenario Reveal is calibrated to test a client condition the baseline may not absorb. Document what was sold or reduced, what was bought or increased, old and new weights, dollar impact, rationale, and the trade-off. If the result is unexpectedly PASS, stop and report it to the instructor; do not skip the checkpoint.</x:v>
       </x:c>
       <x:c r="B38" s="50"/>
       <x:c r="C38" s="50"/>
@@ -5735,7 +5875,7 @@
     </x:row>
     <x:row r="39" ht="18" hidden="0" customHeight="1">
       <x:c r="A39" s="51" t="s">
-        <x:v>92</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="B39" s="51"/>
       <x:c r="C39" s="51"/>
@@ -5750,22 +5890,22 @@
     </x:row>
     <x:row r="40" ht="30" hidden="0" customHeight="1">
       <x:c r="B40" s="25" t="s">
-        <x:v>93</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C40" s="25" t="s">
-        <x:v>94</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="D40" s="25" t="s">
-        <x:v>95</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="E40" s="25" t="s">
-        <x:v>96</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="F40" s="25" t="s">
-        <x:v>97</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="G40" s="26" t="s">
-        <x:v>98</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="H40" s="26"/>
       <x:c r="I40" s="26"/>
@@ -5858,7 +5998,7 @@
     </x:row>
     <x:row r="47" ht="21.75" hidden="0" customHeight="1">
       <x:c r="A47" s="52" t="s">
-        <x:v>99</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="B47" s="52"/>
       <x:c r="C47" s="52"/>
@@ -5867,7 +6007,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E47" s="40" t="s">
-        <x:v>100</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="F47" s="40"/>
       <x:c r="G47" s="40"/>
@@ -5878,8 +6018,8 @@
     </x:row>
     <x:row r="48" ht="7.5" hidden="0" customHeight="1"/>
     <x:row r="49" ht="18" hidden="0" customHeight="1">
-      <x:c r="A49" s="51" t="s">
-        <x:v>101</x:v>
+      <x:c r="A49" s="51" t="str">
+        <x:v>  Part B — Revised Scenario Reveal Result  (confirm the corrective portfolio now passes)</x:v>
       </x:c>
       <x:c r="B49" s="51"/>
       <x:c r="C49" s="51"/>
@@ -5893,8 +6033,8 @@
       <x:c r="K49" s="51"/>
     </x:row>
     <x:row r="50" ht="31.5" hidden="0" customHeight="1">
-      <x:c r="A50" s="8" t="s">
-        <x:v>102</x:v>
+      <x:c r="A50" s="8" t="str">
+        <x:v>Using the new weights from Part A, recalculate the released scenario result. The result must be at or above the IPS Tripwire. Show the calculation clearly and retain the baseline evidence separately.</x:v>
       </x:c>
       <x:c r="B50" s="8"/>
       <x:c r="C50" s="8"/>
@@ -5909,22 +6049,22 @@
     </x:row>
     <x:row r="51" ht="30" hidden="0" customHeight="1">
       <x:c r="B51" s="25" t="s">
-        <x:v>47</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C51" s="25" t="s">
-        <x:v>103</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="D51" s="25" t="s">
-        <x:v>104</x:v>
-      </x:c>
-      <x:c r="E51" s="25" t="s">
-        <x:v>105</x:v>
-      </x:c>
-      <x:c r="F51" s="25" t="s">
-        <x:v>106</x:v>
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="E51" s="25" t="str">
+        <x:v>Scenario Reveal E(R)</x:v>
+      </x:c>
+      <x:c r="F51" s="25" t="str">
+        <x:v>Wtd Scenario Contribution</x:v>
       </x:c>
       <x:c r="G51" s="26" t="s">
-        <x:v>107</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="H51" s="26"/>
       <x:c r="I51" s="26"/>
@@ -5933,7 +6073,7 @@
     </x:row>
     <x:row r="52" ht="21.75" hidden="0" customHeight="1">
       <x:c r="B52" s="27" t="s">
-        <x:v>51</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="C52" s="21"/>
       <x:c r="D52" s="31" t="str">
@@ -5956,7 +6096,7 @@
     </x:row>
     <x:row r="53" ht="21.75" hidden="0" customHeight="1">
       <x:c r="B53" s="29" t="s">
-        <x:v>52</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C53" s="21"/>
       <x:c r="D53" s="31" t="str">
@@ -5979,7 +6119,7 @@
     </x:row>
     <x:row r="54" ht="21.75" hidden="0" customHeight="1">
       <x:c r="B54" s="27" t="s">
-        <x:v>53</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C54" s="21"/>
       <x:c r="D54" s="31" t="str">
@@ -6002,7 +6142,7 @@
     </x:row>
     <x:row r="55" ht="24" hidden="0" customHeight="1">
       <x:c r="A55" s="38" t="s">
-        <x:v>108</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="B55" s="38"/>
       <x:c r="C55" s="32" t="n">
@@ -6025,7 +6165,7 @@
     </x:row>
     <x:row r="56" ht="25.5" hidden="0" customHeight="1">
       <x:c r="B56" s="10" t="s">
-        <x:v>109</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C56" s="32" t="n">
         <x:f aca="0">$G$5</x:f>
@@ -6042,8 +6182,8 @@
       <x:c r="F56" s="46" t="str">
         <x:f aca="0">IF(D56="","",IF(D56&gt;=$G$5,"✓ REVISED PASS","✗ STILL FAILING — ADJUST FURTHER"))</x:f>
       </x:c>
-      <x:c r="G56" s="48" t="s">
-        <x:v>110</x:v>
+      <x:c r="G56" s="48" t="str">
+        <x:v>Revised Scenario Reveal return must be ≥ IPS Tripwire (G5). If still failing, make a further documented adjustment and re-test.</x:v>
       </x:c>
       <x:c r="H56" s="48"/>
       <x:c r="I56" s="48"/>
@@ -6052,8 +6192,8 @@
     </x:row>
     <x:row r="57" ht="7.5" hidden="0" customHeight="1"/>
     <x:row r="58" ht="19.5" hidden="0" customHeight="1">
-      <x:c r="A58" s="4" t="s">
-        <x:v>111</x:v>
+      <x:c r="A58" s="4" t="str">
+        <x:v>  SECTION 6 — FINAL RISK METRICS SUMMARY  (for Gate 2 submission)</x:v>
       </x:c>
       <x:c r="B58" s="4"/>
       <x:c r="C58" s="4"/>
@@ -6068,7 +6208,7 @@
     </x:row>
     <x:row r="59" ht="31.5" hidden="0" customHeight="1">
       <x:c r="A59" s="8" t="str">
-        <x:v>These are the final numbers your team submits. If you re-allocated in Section 5, use the revised portfolio metrics here. If the original portfolio passed, carry forward the verified Phase 2 metrics.</x:v>
+        <x:v>These are the final Gate 2 numbers. Use the revised portfolio metrics after the Scenario Reveal remediation and retain the pre-reveal baseline snapshot as a separate submitted record.</x:v>
       </x:c>
       <x:c r="B59" s="8"/>
       <x:c r="C59" s="8"/>
@@ -6083,16 +6223,16 @@
     </x:row>
     <x:row r="60" ht="30" hidden="0" customHeight="1">
       <x:c r="B60" s="25" t="s">
-        <x:v>28</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C60" s="25" t="s">
-        <x:v>112</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="D60" s="25" t="s">
-        <x:v>113</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="E60" s="26" t="s">
-        <x:v>114</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="F60" s="26"/>
       <x:c r="G60" s="26"/>
@@ -6103,11 +6243,11 @@
     </x:row>
     <x:row r="61" ht="24" hidden="0" customHeight="1">
       <x:c r="B61" s="10" t="s">
-        <x:v>36</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C61" s="42"/>
       <x:c r="D61" s="55" t="s">
-        <x:v>115</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="E61" s="44" t="str">
         <x:v>Weighted average β from the Phase 2 security-selection record</x:v>
@@ -6121,7 +6261,7 @@
     </x:row>
     <x:row r="62" ht="24" hidden="0" customHeight="1">
       <x:c r="B62" s="12" t="s">
-        <x:v>69</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="C62" s="21"/>
       <x:c r="D62" s="55" t="str">
@@ -6139,14 +6279,14 @@
     </x:row>
     <x:row r="63" ht="24" hidden="0" customHeight="1">
       <x:c r="B63" s="10" t="s">
-        <x:v>116</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C63" s="42"/>
       <x:c r="D63" s="55" t="s">
-        <x:v>117</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="E63" s="44" t="s">
-        <x:v>118</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F63" s="44"/>
       <x:c r="G63" s="44"/>
@@ -6156,15 +6296,15 @@
       <x:c r="K63" s="44"/>
     </x:row>
     <x:row r="64" ht="24" hidden="0" customHeight="1">
-      <x:c r="B64" s="12" t="s">
-        <x:v>33</x:v>
+      <x:c r="B64" s="12" t="str">
+        <x:v>Scenario Reveal Portfolio Return</x:v>
       </x:c>
       <x:c r="C64" s="21"/>
       <x:c r="D64" s="55" t="s">
-        <x:v>119</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="E64" s="44" t="s">
-        <x:v>120</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="F64" s="44"/>
       <x:c r="G64" s="44"/>
@@ -6174,15 +6314,15 @@
       <x:c r="K64" s="44"/>
     </x:row>
     <x:row r="65" ht="24" hidden="0" customHeight="1">
-      <x:c r="B65" s="10" t="s">
-        <x:v>121</x:v>
+      <x:c r="B65" s="10" t="str">
+        <x:v>Scenario Reveal $ P&amp;L</x:v>
       </x:c>
       <x:c r="C65" s="56"/>
       <x:c r="D65" s="55" t="s">
-        <x:v>122</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="E65" s="44" t="s">
-        <x:v>120</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="F65" s="44"/>
       <x:c r="G65" s="44"/>
@@ -6192,15 +6332,15 @@
       <x:c r="K65" s="44"/>
     </x:row>
     <x:row r="66" ht="24" hidden="0" customHeight="1">
-      <x:c r="B66" s="12" t="s">
-        <x:v>123</x:v>
+      <x:c r="B66" s="12" t="str">
+        <x:v>IPS Mandate Status after re-test</x:v>
       </x:c>
       <x:c r="C66" s="57"/>
       <x:c r="D66" s="55" t="s">
-        <x:v>124</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="E66" s="44" t="s">
-        <x:v>125</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="F66" s="44"/>
       <x:c r="G66" s="44"/>
@@ -6212,7 +6352,7 @@
     <x:row r="68" ht="7.5" hidden="0" customHeight="1"/>
     <x:row r="69" ht="19.5" hidden="0" customHeight="1">
       <x:c r="A69" s="4" t="s">
-        <x:v>126</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="B69" s="4"/>
       <x:c r="C69" s="4"/>
@@ -6227,10 +6367,10 @@
     </x:row>
     <x:row r="70" ht="18" hidden="0" customHeight="1">
       <x:c r="B70" s="58" t="s">
-        <x:v>127</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C70" s="7" t="s">
-        <x:v>128</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="D70" s="7"/>
       <x:c r="E70" s="7"/>
@@ -6243,10 +6383,10 @@
     </x:row>
     <x:row r="71" ht="18" hidden="0" customHeight="1">
       <x:c r="B71" s="59" t="s">
-        <x:v>127</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C71" s="7" t="s">
-        <x:v>129</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="D71" s="7"/>
       <x:c r="E71" s="7"/>
@@ -6259,10 +6399,10 @@
     </x:row>
     <x:row r="72" ht="18" hidden="0" customHeight="1">
       <x:c r="B72" s="60" t="s">
-        <x:v>127</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C72" s="7" t="s">
-        <x:v>130</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="D72" s="7"/>
       <x:c r="E72" s="7"/>
@@ -6275,10 +6415,10 @@
     </x:row>
     <x:row r="73" ht="18" hidden="0" customHeight="1">
       <x:c r="B73" s="61" t="s">
-        <x:v>127</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C73" s="7" t="s">
-        <x:v>131</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="D73" s="7"/>
       <x:c r="E73" s="7"/>
@@ -6291,10 +6431,10 @@
     </x:row>
     <x:row r="74" ht="18" hidden="0" customHeight="1">
       <x:c r="B74" s="62" t="s">
-        <x:v>127</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C74" s="7" t="s">
-        <x:v>132</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="D74" s="7"/>
       <x:c r="E74" s="7"/>
@@ -6307,10 +6447,10 @@
     </x:row>
     <x:row r="75" ht="18" hidden="0" customHeight="1">
       <x:c r="B75" s="63" t="s">
-        <x:v>127</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C75" s="7" t="s">
-        <x:v>133</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="D75" s="7"/>
       <x:c r="E75" s="7"/>
@@ -6388,6 +6528,7 @@
     <x:mergeCell ref="C73:K73"/>
     <x:mergeCell ref="C74:K74"/>
     <x:mergeCell ref="C75:K75"/>
+    <x:mergeCell ref="I6:J6"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="C20:C20">
     <x:cfRule type="cellIs" dxfId="0" priority="2" aboveAverage="0" percent="0" bottom="0" operator="equal" rank="0" equalAverage="0">
@@ -6436,7 +6577,7 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R651bae8ab1d84fda"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3bd25e4235774f7b"/>
 </x:worksheet>
 </file>
 
@@ -6474,7 +6615,7 @@
     </x:row>
     <x:row r="3" ht="18" hidden="0" customHeight="1">
       <x:c r="A3" s="3" t="str">
-        <x:v>BUS 331 Investments  |  Endicott College  |  Apply the approved Phase 1 Bear Case to the Phase 2 Portfolio</x:v>
+        <x:v>BUS 331 Investments | Stage 1: submit baseline; Stage 2: run the instructor-issued Scenario Reveal and remediation test</x:v>
       </x:c>
       <x:c r="B3" s="3"/>
       <x:c r="C3" s="3"/>
@@ -6490,33 +6631,39 @@
     <x:row r="4" ht="6" hidden="0" customHeight="1"/>
     <x:row r="5" ht="21.75" hidden="0" customHeight="1">
       <x:c r="B5" s="17" t="s">
-        <x:v>40</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C5" s="18"/>
       <x:c r="D5" s="17" t="s">
-        <x:v>41</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="E5" s="19" t="n">
         <x:v>500000</x:v>
       </x:c>
       <x:c r="F5" s="20" t="s">
-        <x:v>42</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="G5" s="21"/>
       <x:c r="H5" s="17" t="s">
-        <x:v>43</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="I5" s="22" t="str">
         <x:v>(from Phase 1)</x:v>
       </x:c>
       <x:c r="J5" s="23" t="s">
-        <x:v>44</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="6" hidden="0" customHeight="1"/>
+        <x:v>18</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="6" hidden="0" customHeight="1">
+      <x:c r="H6" s="99" t="str">
+        <x:v>Scenario Release Packet ID:</x:v>
+      </x:c>
+      <x:c r="I6" s="99" t="str"/>
+      <x:c r="J6" s="99"/>
+    </x:row>
     <x:row r="7" ht="19.5" hidden="0" customHeight="1">
-      <x:c r="A7" s="4" t="s">
-        <x:v>45</x:v>
+      <x:c r="A7" s="4" t="str">
+        <x:v>  SECTION 1 — SCENARIO REVEAL ASSUMPTIONS  (enter only after instructor release)</x:v>
       </x:c>
       <x:c r="B7" s="4"/>
       <x:c r="C7" s="4"/>
@@ -6530,8 +6677,8 @@
       <x:c r="K7" s="4"/>
     </x:row>
     <x:row r="8" ht="31.5" hidden="0" customHeight="1">
-      <x:c r="A8" s="24" t="s">
-        <x:v>46</x:v>
+      <x:c r="A8" s="24" t="str">
+        <x:v>Stage 1: submit the baseline portfolio snapshot using your approved Phase 1 bear-case inputs. Stage 2: after the instructor issues a Scenario Reveal packet, copy the released inputs below exactly. These values drive the remediation test; do not soften them, change the client mandate, or enter values before the release.</x:v>
       </x:c>
       <x:c r="B8" s="24"/>
       <x:c r="C8" s="24"/>
@@ -6545,17 +6692,19 @@
       <x:c r="K8" s="24"/>
     </x:row>
     <x:row r="9" ht="30" hidden="0" customHeight="1">
-      <x:c r="B9" s="25" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="C9" s="25" t="s">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="D9" s="25" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="E9" s="26" t="s">
-        <x:v>50</x:v>
+      <x:c r="B9" s="25" t="str">
+        <x:v>Asset Class</x:v>
+      </x:c>
+      <x:c r="C9" s="25" t="str">
+        <x:v>Scenario Reveal
+E(R) Input</x:v>
+      </x:c>
+      <x:c r="D9" s="25" t="str">
+        <x:v>Scenario Reveal
+Std Dev (σ)</x:v>
+      </x:c>
+      <x:c r="E9" s="26" t="str">
+        <x:v>Instructor packet / source reference</x:v>
       </x:c>
       <x:c r="F9" s="26"/>
       <x:c r="G9" s="26"/>
@@ -6566,7 +6715,7 @@
     </x:row>
     <x:row r="10" ht="21.75" hidden="0" customHeight="1">
       <x:c r="B10" s="27" t="s">
-        <x:v>51</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="C10" s="21"/>
       <x:c r="D10" s="21"/>
@@ -6580,7 +6729,7 @@
     </x:row>
     <x:row r="11" ht="21.75" hidden="0" customHeight="1">
       <x:c r="B11" s="29" t="s">
-        <x:v>52</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C11" s="21"/>
       <x:c r="D11" s="21"/>
@@ -6594,7 +6743,7 @@
     </x:row>
     <x:row r="12" ht="21.75" hidden="0" customHeight="1">
       <x:c r="B12" s="27" t="s">
-        <x:v>53</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C12" s="21"/>
       <x:c r="D12" s="21"/>
@@ -6609,7 +6758,7 @@
     <x:row r="13" ht="7.5" hidden="0" customHeight="1"/>
     <x:row r="14" ht="19.5" hidden="0" customHeight="1">
       <x:c r="A14" s="4" t="str">
-        <x:v>  SECTION 2 — BASE CASE PORTFOLIO  (enter Phase 2 Workstream A weights)</x:v>
+        <x:v>  SECTION 2 — BASELINE PORTFOLIO  (submitted before Scenario Reveal)</x:v>
       </x:c>
       <x:c r="B14" s="4"/>
       <x:c r="C14" s="4"/>
@@ -6624,7 +6773,7 @@
     </x:row>
     <x:row r="15" ht="31.5" hidden="0" customHeight="1">
       <x:c r="A15" s="8" t="str">
-        <x:v>Enter the Solver-supported weights from Phase 2 Workstream A for this client. Weights must sum to 100%. The Base Case return and risk metrics auto-calculate.</x:v>
+        <x:v>Enter the Solver-supported baseline weights from Workstream A and submit the baseline snapshot before the Scenario Reveal. Keep that original evidence in Canvas. Do not overwrite the submitted allocation after the release; document all changes in Section 5.</x:v>
       </x:c>
       <x:c r="B15" s="8"/>
       <x:c r="C15" s="8"/>
@@ -6639,36 +6788,39 @@
     </x:row>
     <x:row r="16" ht="33.75" hidden="0" customHeight="1">
       <x:c r="B16" s="25" t="s">
-        <x:v>47</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C16" s="25" t="str">
         <x:v>Weight
 (Workstream A)</x:v>
       </x:c>
       <x:c r="D16" s="25" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="E16" s="25" t="s">
-        <x:v>55</x:v>
-      </x:c>
-      <x:c r="F16" s="25" t="s">
-        <x:v>56</x:v>
-      </x:c>
-      <x:c r="G16" s="25" t="s">
-        <x:v>57</x:v>
+        <x:v>23</x:v>
+      </x:c>
+      <x:c r="E16" s="25" t="str">
+        <x:v>Baseline Case
+E(R) Contrib.</x:v>
+      </x:c>
+      <x:c r="F16" s="25" t="str">
+        <x:v>Scenario Reveal
+Return Contrib.</x:v>
+      </x:c>
+      <x:c r="G16" s="25" t="str">
+        <x:v>Scenario Reveal
+$ P&amp;L</x:v>
       </x:c>
       <x:c r="H16" s="25" t="s">
-        <x:v>58</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="I16" s="30" t="s">
-        <x:v>59</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="J16" s="30"/>
       <x:c r="K16" s="30"/>
     </x:row>
     <x:row r="17" ht="21.75" hidden="0" customHeight="1">
       <x:c r="B17" s="27" t="s">
-        <x:v>51</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="C17" s="21"/>
       <x:c r="D17" s="31" t="str">
@@ -6688,7 +6840,7 @@
     </x:row>
     <x:row r="18" ht="21.75" hidden="0" customHeight="1">
       <x:c r="B18" s="29" t="s">
-        <x:v>52</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C18" s="21"/>
       <x:c r="D18" s="31" t="str">
@@ -6708,7 +6860,7 @@
     </x:row>
     <x:row r="19" ht="21.75" hidden="0" customHeight="1">
       <x:c r="B19" s="27" t="s">
-        <x:v>53</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C19" s="21"/>
       <x:c r="D19" s="31" t="str">
@@ -6728,7 +6880,7 @@
     </x:row>
     <x:row r="20" ht="24" hidden="0" customHeight="1">
       <x:c r="A20" s="38" t="s">
-        <x:v>60</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="B20" s="38"/>
       <x:c r="C20" s="39" t="n">
@@ -6751,8 +6903,8 @@
         <x:f aca="0">IFERROR(SUM(G17:G19),"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="H20" s="40" t="s">
-        <x:v>61</x:v>
+      <x:c r="H20" s="40" t="str">
+        <x:v>← Scenario Reveal return must be ≥ IPS Tripwire (cell G5). See Section 4 verdict below.</x:v>
       </x:c>
       <x:c r="I20" s="40"/>
       <x:c r="J20" s="40"/>
@@ -6760,8 +6912,8 @@
     </x:row>
     <x:row r="21" ht="7.5" hidden="0" customHeight="1"/>
     <x:row r="22" ht="19.5" hidden="0" customHeight="1">
-      <x:c r="A22" s="4" t="s">
-        <x:v>62</x:v>
+      <x:c r="A22" s="4" t="str">
+        <x:v>  SECTION 3 — RISK METRICS  (Baseline &amp; Scenario Reveal)</x:v>
       </x:c>
       <x:c r="B22" s="4"/>
       <x:c r="C22" s="4"/>
@@ -6776,7 +6928,7 @@
     </x:row>
     <x:row r="23" ht="31.5" hidden="0" customHeight="1">
       <x:c r="A23" s="8" t="str">
-        <x:v>Enter portfolio risk metrics for BOTH the Base Case and Bear Case. Beta and σ come from the Phase 2 allocation and selected holdings. Sharpe Ratio is calculated automatically using the formula below.</x:v>
+        <x:v>Enter portfolio risk metrics for the submitted baseline and the Scenario Reveal. Beta and σ come from the Phase 2 allocation and selected holdings. Sharpe Ratio calculates automatically using the formula below.</x:v>
       </x:c>
       <x:c r="B23" s="8"/>
       <x:c r="C23" s="8"/>
@@ -6791,20 +6943,20 @@
     </x:row>
     <x:row r="24" ht="30" hidden="0" customHeight="1">
       <x:c r="B24" s="25" t="s">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="C24" s="25" t="str">
+        <x:v>Baseline
+(Phase 2)</x:v>
+      </x:c>
+      <x:c r="D24" s="25" t="str">
+        <x:v>Scenario Reveal</x:v>
+      </x:c>
+      <x:c r="E24" s="25" t="s">
+        <x:v>27</x:v>
+      </x:c>
+      <x:c r="F24" s="26" t="s">
         <x:v>28</x:v>
-      </x:c>
-      <x:c r="C24" s="25" t="str">
-        <x:v>Base Case
-(Phase 2)</x:v>
-      </x:c>
-      <x:c r="D24" s="25" t="s">
-        <x:v>63</x:v>
-      </x:c>
-      <x:c r="E24" s="25" t="s">
-        <x:v>64</x:v>
-      </x:c>
-      <x:c r="F24" s="26" t="s">
-        <x:v>65</x:v>
       </x:c>
       <x:c r="G24" s="26"/>
       <x:c r="H24" s="26"/>
@@ -6814,11 +6966,11 @@
     </x:row>
     <x:row r="25" ht="21.75" hidden="0" customHeight="1">
       <x:c r="B25" s="17" t="s">
-        <x:v>66</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="C25" s="21"/>
       <x:c r="D25" s="40" t="s">
-        <x:v>67</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="E25" s="40"/>
       <x:c r="F25" s="40"/>
@@ -6830,7 +6982,7 @@
     </x:row>
     <x:row r="26" ht="25.5" hidden="0" customHeight="1">
       <x:c r="B26" s="10" t="s">
-        <x:v>36</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C26" s="41"/>
       <x:c r="D26" s="42"/>
@@ -6838,7 +6990,7 @@
         <x:v>From Phase 2 security selection — weighted average beta of all holdings</x:v>
       </x:c>
       <x:c r="F26" s="44" t="s">
-        <x:v>68</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="G26" s="44"/>
       <x:c r="H26" s="44"/>
@@ -6848,7 +7000,7 @@
     </x:row>
     <x:row r="27" ht="25.5" hidden="0" customHeight="1">
       <x:c r="B27" s="12" t="s">
-        <x:v>69</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="C27" s="21"/>
       <x:c r="D27" s="21"/>
@@ -6856,7 +7008,7 @@
         <x:v>From Phase 2 CME Matrix — portfolio σ from Solver output</x:v>
       </x:c>
       <x:c r="F27" s="44" t="s">
-        <x:v>70</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="G27" s="44"/>
       <x:c r="H27" s="44"/>
@@ -6866,7 +7018,7 @@
     </x:row>
     <x:row r="28" ht="25.5" hidden="0" customHeight="1">
       <x:c r="B28" s="10" t="s">
-        <x:v>71</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="C28" s="41" t="str">
         <x:f aca="0">IFERROR((E20-$C$25)/C27,"")</x:f>
@@ -6875,10 +7027,10 @@
         <x:f aca="0">IFERROR((F20-$C$25)/D27,"")</x:f>
       </x:c>
       <x:c r="E28" s="43" t="s">
-        <x:v>72</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="F28" s="44" t="s">
-        <x:v>73</x:v>
+        <x:v>36</x:v>
       </x:c>
       <x:c r="G28" s="44"/>
       <x:c r="H28" s="44"/>
@@ -6887,21 +7039,21 @@
       <x:c r="K28" s="44"/>
     </x:row>
     <x:row r="29" ht="25.5" hidden="0" customHeight="1">
-      <x:c r="B29" s="12" t="s">
-        <x:v>74</x:v>
+      <x:c r="B29" s="12" t="str">
+        <x:v>Max Drawdown (Scenario Reveal)</x:v>
       </x:c>
       <x:c r="C29" s="45" t="s">
-        <x:v>75</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="D29" s="32" t="n">
         <x:f aca="0">IFERROR(F20,"")</x:f>
         <x:v>0</x:v>
       </x:c>
-      <x:c r="E29" s="43" t="s">
-        <x:v>76</x:v>
-      </x:c>
-      <x:c r="F29" s="44" t="s">
-        <x:v>77</x:v>
+      <x:c r="E29" s="43" t="str">
+        <x:v>Total Scenario Reveal Return (Section 2 row 20)</x:v>
+      </x:c>
+      <x:c r="F29" s="44" t="str">
+        <x:v>Must be ≥ IPS Tripwire (cell G5). This drives the Scenario Reveal verdict.</x:v>
       </x:c>
       <x:c r="G29" s="44"/>
       <x:c r="H29" s="44"/>
@@ -6911,15 +7063,15 @@
     </x:row>
     <x:row r="30" ht="25.5" hidden="0" customHeight="1">
       <x:c r="B30" s="10" t="s">
-        <x:v>78</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="C30" s="42"/>
       <x:c r="D30" s="42"/>
       <x:c r="E30" s="43" t="s">
-        <x:v>79</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="F30" s="44" t="s">
-        <x:v>80</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="G30" s="44"/>
       <x:c r="H30" s="44"/>
@@ -6929,8 +7081,8 @@
     </x:row>
     <x:row r="31" ht="7.5" hidden="0" customHeight="1"/>
     <x:row r="32" ht="19.5" hidden="0" customHeight="1">
-      <x:c r="A32" s="4" t="s">
-        <x:v>81</x:v>
+      <x:c r="A32" s="4" t="str">
+        <x:v>  SECTION 4 — SCENARIO REVEAL VERDICT</x:v>
       </x:c>
       <x:c r="B32" s="4"/>
       <x:c r="C32" s="4"/>
@@ -6945,19 +7097,19 @@
     </x:row>
     <x:row r="33" ht="30" hidden="0" customHeight="1">
       <x:c r="B33" s="25" t="s">
-        <x:v>82</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="C33" s="25" t="s">
-        <x:v>83</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="D33" s="25" t="s">
-        <x:v>84</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="E33" s="25" t="s">
-        <x:v>85</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="F33" s="26" t="s">
-        <x:v>86</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="G33" s="26"/>
       <x:c r="H33" s="26"/>
@@ -6967,7 +7119,7 @@
     </x:row>
     <x:row r="34" ht="25.5" hidden="0" customHeight="1">
       <x:c r="B34" s="10" t="s">
-        <x:v>87</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="C34" s="32" t="n">
         <x:f aca="0">$G$5</x:f>
@@ -6985,7 +7137,7 @@
         <x:f aca="0">IF(D34="","",IF(D34&gt;=C34,"✓ PASS","✗ FAIL — RE-ALLOCATE"))</x:f>
       </x:c>
       <x:c r="G34" s="47" t="str">
-        <x:f aca="0">IF(D34="","",IF(D34&gt;=C34,"Portfolio passes IPS mandate. No re-allocation required. Proceed to Section 6 (Final Metrics).","FAIL: Portfolio breaches IPS Tripwire by "&amp;TEXT(ABS(D34-C34),"0.0%")&amp;". Complete Section 5 (Re-allocation) to bring portfolio within mandate before submitting."))</x:f>
+        <x:f aca="0">IF(D34="","",IF(D34&gt;=C34,"Scenario Reveal shows PASS. Stop and report this result to the instructor; do not use a PASS to skip the remediation checkpoint.","BREACH: Portfolio misses the IPS Tripwire by "&amp;TEXT(ABS(D34-C34),"0.0%")&amp;". Complete Section 5 with a real trade, trade-off, and full re-test before Gate 2."))</x:f>
       </x:c>
       <x:c r="H34" s="47"/>
       <x:c r="I34" s="47"/>
@@ -6994,7 +7146,7 @@
     </x:row>
     <x:row r="35" ht="25.5" hidden="0" customHeight="1">
       <x:c r="B35" s="12" t="s">
-        <x:v>88</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C35" s="21"/>
       <x:c r="D35" s="32" t="str">
@@ -7008,17 +7160,21 @@
         <x:f aca="0">IF(D35="","",IF(D35&lt;=C35,"✓ PASS","✗ EXCEED"))</x:f>
       </x:c>
       <x:c r="G35" s="48" t="s">
-        <x:v>89</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="H35" s="48"/>
       <x:c r="I35" s="48"/>
       <x:c r="J35" s="48"/>
       <x:c r="K35" s="48"/>
     </x:row>
-    <x:row r="36" ht="7.5" hidden="0" customHeight="1"/>
+    <x:row r="36" ht="7.5" hidden="0" customHeight="1">
+      <x:c r="A36" t="str">
+        <x:v>  SECTION 5 — REQUIRED REMEDIATION &amp; RE-TEST</x:v>
+      </x:c>
+    </x:row>
     <x:row r="37" ht="19.5" hidden="0" customHeight="1">
-      <x:c r="A37" s="49" t="s">
-        <x:v>90</x:v>
+      <x:c r="A37" s="49" t="str">
+        <x:v>  A breach requires a real portfolio change, stated trade-off, and full re-test</x:v>
       </x:c>
       <x:c r="B37" s="49"/>
       <x:c r="C37" s="49"/>
@@ -7032,8 +7188,8 @@
       <x:c r="K37" s="49"/>
     </x:row>
     <x:row r="38" ht="31.5" hidden="0" customHeight="1">
-      <x:c r="A38" s="50" t="s">
-        <x:v>91</x:v>
+      <x:c r="A38" s="50" t="str">
+        <x:v>The Scenario Reveal is calibrated to test a client condition the baseline may not absorb. Document what was sold or reduced, what was bought or increased, old and new weights, dollar impact, rationale, and the trade-off. If the result is unexpectedly PASS, stop and report it to the instructor; do not skip the checkpoint.</x:v>
       </x:c>
       <x:c r="B38" s="50"/>
       <x:c r="C38" s="50"/>
@@ -7048,7 +7204,7 @@
     </x:row>
     <x:row r="39" ht="18" hidden="0" customHeight="1">
       <x:c r="A39" s="51" t="s">
-        <x:v>92</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="B39" s="51"/>
       <x:c r="C39" s="51"/>
@@ -7063,22 +7219,22 @@
     </x:row>
     <x:row r="40" ht="30" hidden="0" customHeight="1">
       <x:c r="B40" s="25" t="s">
-        <x:v>93</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C40" s="25" t="s">
-        <x:v>94</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="D40" s="25" t="s">
-        <x:v>95</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="E40" s="25" t="s">
-        <x:v>96</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="F40" s="25" t="s">
-        <x:v>97</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="G40" s="26" t="s">
-        <x:v>98</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="H40" s="26"/>
       <x:c r="I40" s="26"/>
@@ -7171,7 +7327,7 @@
     </x:row>
     <x:row r="47" ht="21.75" hidden="0" customHeight="1">
       <x:c r="A47" s="52" t="s">
-        <x:v>99</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="B47" s="52"/>
       <x:c r="C47" s="52"/>
@@ -7180,7 +7336,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E47" s="40" t="s">
-        <x:v>100</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="F47" s="40"/>
       <x:c r="G47" s="40"/>
@@ -7191,8 +7347,8 @@
     </x:row>
     <x:row r="48" ht="7.5" hidden="0" customHeight="1"/>
     <x:row r="49" ht="18" hidden="0" customHeight="1">
-      <x:c r="A49" s="51" t="s">
-        <x:v>101</x:v>
+      <x:c r="A49" s="51" t="str">
+        <x:v>  Part B — Revised Scenario Reveal Result  (confirm the corrective portfolio now passes)</x:v>
       </x:c>
       <x:c r="B49" s="51"/>
       <x:c r="C49" s="51"/>
@@ -7206,8 +7362,8 @@
       <x:c r="K49" s="51"/>
     </x:row>
     <x:row r="50" ht="31.5" hidden="0" customHeight="1">
-      <x:c r="A50" s="8" t="s">
-        <x:v>102</x:v>
+      <x:c r="A50" s="8" t="str">
+        <x:v>Using the new weights from Part A, recalculate the released scenario result. The result must be at or above the IPS Tripwire. Show the calculation clearly and retain the baseline evidence separately.</x:v>
       </x:c>
       <x:c r="B50" s="8"/>
       <x:c r="C50" s="8"/>
@@ -7222,22 +7378,22 @@
     </x:row>
     <x:row r="51" ht="30" hidden="0" customHeight="1">
       <x:c r="B51" s="25" t="s">
-        <x:v>47</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="C51" s="25" t="s">
-        <x:v>103</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="D51" s="25" t="s">
-        <x:v>104</x:v>
-      </x:c>
-      <x:c r="E51" s="25" t="s">
-        <x:v>105</x:v>
-      </x:c>
-      <x:c r="F51" s="25" t="s">
-        <x:v>106</x:v>
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="E51" s="25" t="str">
+        <x:v>Scenario Reveal E(R)</x:v>
+      </x:c>
+      <x:c r="F51" s="25" t="str">
+        <x:v>Wtd Scenario Contribution</x:v>
       </x:c>
       <x:c r="G51" s="26" t="s">
-        <x:v>107</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="H51" s="26"/>
       <x:c r="I51" s="26"/>
@@ -7246,7 +7402,7 @@
     </x:row>
     <x:row r="52" ht="21.75" hidden="0" customHeight="1">
       <x:c r="B52" s="27" t="s">
-        <x:v>51</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="C52" s="21"/>
       <x:c r="D52" s="31" t="str">
@@ -7269,7 +7425,7 @@
     </x:row>
     <x:row r="53" ht="21.75" hidden="0" customHeight="1">
       <x:c r="B53" s="29" t="s">
-        <x:v>52</x:v>
+        <x:v>20</x:v>
       </x:c>
       <x:c r="C53" s="21"/>
       <x:c r="D53" s="31" t="str">
@@ -7292,7 +7448,7 @@
     </x:row>
     <x:row r="54" ht="21.75" hidden="0" customHeight="1">
       <x:c r="B54" s="27" t="s">
-        <x:v>53</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="C54" s="21"/>
       <x:c r="D54" s="31" t="str">
@@ -7315,7 +7471,7 @@
     </x:row>
     <x:row r="55" ht="24" hidden="0" customHeight="1">
       <x:c r="A55" s="38" t="s">
-        <x:v>108</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="B55" s="38"/>
       <x:c r="C55" s="32" t="n">
@@ -7338,7 +7494,7 @@
     </x:row>
     <x:row r="56" ht="25.5" hidden="0" customHeight="1">
       <x:c r="B56" s="10" t="s">
-        <x:v>109</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C56" s="32" t="n">
         <x:f aca="0">$G$5</x:f>
@@ -7355,8 +7511,8 @@
       <x:c r="F56" s="46" t="str">
         <x:f aca="0">IF(D56="","",IF(D56&gt;=$G$5,"✓ REVISED PASS","✗ STILL FAILING — ADJUST FURTHER"))</x:f>
       </x:c>
-      <x:c r="G56" s="48" t="s">
-        <x:v>110</x:v>
+      <x:c r="G56" s="48" t="str">
+        <x:v>Revised Scenario Reveal return must be ≥ IPS Tripwire (G5). If still failing, make a further documented adjustment and re-test.</x:v>
       </x:c>
       <x:c r="H56" s="48"/>
       <x:c r="I56" s="48"/>
@@ -7365,8 +7521,8 @@
     </x:row>
     <x:row r="57" ht="7.5" hidden="0" customHeight="1"/>
     <x:row r="58" ht="19.5" hidden="0" customHeight="1">
-      <x:c r="A58" s="4" t="s">
-        <x:v>111</x:v>
+      <x:c r="A58" s="4" t="str">
+        <x:v>  SECTION 6 — FINAL RISK METRICS SUMMARY  (for Gate 2 submission)</x:v>
       </x:c>
       <x:c r="B58" s="4"/>
       <x:c r="C58" s="4"/>
@@ -7381,7 +7537,7 @@
     </x:row>
     <x:row r="59" ht="31.5" hidden="0" customHeight="1">
       <x:c r="A59" s="8" t="str">
-        <x:v>These are the final numbers your team submits. If you re-allocated in Section 5, use the revised portfolio metrics here. If the original portfolio passed, carry forward the verified Phase 2 metrics.</x:v>
+        <x:v>These are the final Gate 2 numbers. Use the revised portfolio metrics after the Scenario Reveal remediation and retain the pre-reveal baseline snapshot as a separate submitted record.</x:v>
       </x:c>
       <x:c r="B59" s="8"/>
       <x:c r="C59" s="8"/>
@@ -7396,16 +7552,16 @@
     </x:row>
     <x:row r="60" ht="30" hidden="0" customHeight="1">
       <x:c r="B60" s="25" t="s">
-        <x:v>28</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="C60" s="25" t="s">
-        <x:v>112</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="D60" s="25" t="s">
-        <x:v>113</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="E60" s="26" t="s">
-        <x:v>114</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="F60" s="26"/>
       <x:c r="G60" s="26"/>
@@ -7416,11 +7572,11 @@
     </x:row>
     <x:row r="61" ht="24" hidden="0" customHeight="1">
       <x:c r="B61" s="10" t="s">
-        <x:v>36</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C61" s="42"/>
       <x:c r="D61" s="55" t="s">
-        <x:v>115</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="E61" s="44" t="str">
         <x:v>Weighted average β from the Phase 2 security-selection record</x:v>
@@ -7434,7 +7590,7 @@
     </x:row>
     <x:row r="62" ht="24" hidden="0" customHeight="1">
       <x:c r="B62" s="12" t="s">
-        <x:v>69</x:v>
+        <x:v>32</x:v>
       </x:c>
       <x:c r="C62" s="21"/>
       <x:c r="D62" s="55" t="str">
@@ -7452,14 +7608,14 @@
     </x:row>
     <x:row r="63" ht="24" hidden="0" customHeight="1">
       <x:c r="B63" s="10" t="s">
-        <x:v>116</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="C63" s="42"/>
       <x:c r="D63" s="55" t="s">
-        <x:v>117</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="E63" s="44" t="s">
-        <x:v>118</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="F63" s="44"/>
       <x:c r="G63" s="44"/>
@@ -7469,15 +7625,15 @@
       <x:c r="K63" s="44"/>
     </x:row>
     <x:row r="64" ht="24" hidden="0" customHeight="1">
-      <x:c r="B64" s="12" t="s">
-        <x:v>33</x:v>
+      <x:c r="B64" s="12" t="str">
+        <x:v>Scenario Reveal Portfolio Return</x:v>
       </x:c>
       <x:c r="C64" s="21"/>
       <x:c r="D64" s="55" t="s">
-        <x:v>119</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="E64" s="44" t="s">
-        <x:v>120</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="F64" s="44"/>
       <x:c r="G64" s="44"/>
@@ -7487,15 +7643,15 @@
       <x:c r="K64" s="44"/>
     </x:row>
     <x:row r="65" ht="24" hidden="0" customHeight="1">
-      <x:c r="B65" s="10" t="s">
-        <x:v>121</x:v>
+      <x:c r="B65" s="10" t="str">
+        <x:v>Scenario Reveal $ P&amp;L</x:v>
       </x:c>
       <x:c r="C65" s="56"/>
       <x:c r="D65" s="55" t="s">
-        <x:v>122</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="E65" s="44" t="s">
-        <x:v>120</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="F65" s="44"/>
       <x:c r="G65" s="44"/>
@@ -7505,15 +7661,15 @@
       <x:c r="K65" s="44"/>
     </x:row>
     <x:row r="66" ht="24" hidden="0" customHeight="1">
-      <x:c r="B66" s="12" t="s">
-        <x:v>123</x:v>
+      <x:c r="B66" s="12" t="str">
+        <x:v>IPS Mandate Status after re-test</x:v>
       </x:c>
       <x:c r="C66" s="57"/>
       <x:c r="D66" s="55" t="s">
-        <x:v>124</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="E66" s="44" t="s">
-        <x:v>125</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="F66" s="44"/>
       <x:c r="G66" s="44"/>
@@ -7525,7 +7681,7 @@
     <x:row r="68" ht="7.5" hidden="0" customHeight="1"/>
     <x:row r="69" ht="19.5" hidden="0" customHeight="1">
       <x:c r="A69" s="4" t="s">
-        <x:v>126</x:v>
+        <x:v>75</x:v>
       </x:c>
       <x:c r="B69" s="4"/>
       <x:c r="C69" s="4"/>
@@ -7540,10 +7696,10 @@
     </x:row>
     <x:row r="70" ht="18" hidden="0" customHeight="1">
       <x:c r="B70" s="58" t="s">
-        <x:v>127</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C70" s="7" t="s">
-        <x:v>128</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="D70" s="7"/>
       <x:c r="E70" s="7"/>
@@ -7556,10 +7712,10 @@
     </x:row>
     <x:row r="71" ht="18" hidden="0" customHeight="1">
       <x:c r="B71" s="59" t="s">
-        <x:v>127</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C71" s="7" t="s">
-        <x:v>129</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="D71" s="7"/>
       <x:c r="E71" s="7"/>
@@ -7572,10 +7728,10 @@
     </x:row>
     <x:row r="72" ht="18" hidden="0" customHeight="1">
       <x:c r="B72" s="60" t="s">
-        <x:v>127</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C72" s="7" t="s">
-        <x:v>130</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="D72" s="7"/>
       <x:c r="E72" s="7"/>
@@ -7588,10 +7744,10 @@
     </x:row>
     <x:row r="73" ht="18" hidden="0" customHeight="1">
       <x:c r="B73" s="61" t="s">
-        <x:v>127</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C73" s="7" t="s">
-        <x:v>131</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="D73" s="7"/>
       <x:c r="E73" s="7"/>
@@ -7604,10 +7760,10 @@
     </x:row>
     <x:row r="74" ht="18" hidden="0" customHeight="1">
       <x:c r="B74" s="62" t="s">
-        <x:v>127</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C74" s="7" t="s">
-        <x:v>132</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="D74" s="7"/>
       <x:c r="E74" s="7"/>
@@ -7620,10 +7776,10 @@
     </x:row>
     <x:row r="75" ht="18" hidden="0" customHeight="1">
       <x:c r="B75" s="63" t="s">
-        <x:v>127</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="C75" s="7" t="s">
-        <x:v>133</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="D75" s="7"/>
       <x:c r="E75" s="7"/>
@@ -7701,6 +7857,7 @@
     <x:mergeCell ref="C73:K73"/>
     <x:mergeCell ref="C74:K74"/>
     <x:mergeCell ref="C75:K75"/>
+    <x:mergeCell ref="I6:J6"/>
   </x:mergeCells>
   <x:conditionalFormatting sqref="C20:C20">
     <x:cfRule type="cellIs" dxfId="0" priority="2" aboveAverage="0" percent="0" bottom="0" operator="equal" rank="0" equalAverage="0">
@@ -7749,6 +7906,359 @@
     </x:dataValidation>
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Ra4eee8eb9e7744d2"/>
+  <x:legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2ecc168ba35c43f4"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="14" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="15" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="28" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="34" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="28" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="30" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="66" t="str">
+        <x:v>Phase 2 · Scenario Reveal &amp; Required Remediation</x:v>
+      </x:c>
+      <x:c r="B1" s="66"/>
+      <x:c r="C1" s="66"/>
+      <x:c r="D1" s="66"/>
+      <x:c r="E1" s="66"/>
+      <x:c r="F1" s="66"/>
+      <x:c r="G1" s="66"/>
+      <x:c r="H1" s="66"/>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="68" t="str">
+        <x:v>BUS331 Investments | Use this tab only after the instructor releases the client-specific adverse-event packet.</x:v>
+      </x:c>
+      <x:c r="B2" s="68"/>
+      <x:c r="C2" s="68"/>
+      <x:c r="D2" s="68"/>
+      <x:c r="E2" s="68"/>
+      <x:c r="F2" s="68"/>
+      <x:c r="G2" s="68"/>
+      <x:c r="H2" s="68"/>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="72" t="str">
+        <x:v>Purpose</x:v>
+      </x:c>
+      <x:c r="B5" s="73"/>
+      <x:c r="C5" s="73"/>
+      <x:c r="D5" s="73"/>
+      <x:c r="E5" s="73"/>
+      <x:c r="F5" s="73"/>
+      <x:c r="G5" s="73"/>
+      <x:c r="H5" s="74"/>
+    </x:row>
+    <x:row r="6" ht="30" customHeight="1">
+      <x:c r="A6" s="79" t="str">
+        <x:v>Your committee first submits a baseline portfolio snapshot. The instructor then releases an adverse-event scenario calibrated to test a named client goal, constraint, or tripwire. The reveal is intentionally not included in this public template.</x:v>
+      </x:c>
+      <x:c r="B6" s="80"/>
+      <x:c r="C6" s="80"/>
+      <x:c r="D6" s="80"/>
+      <x:c r="E6" s="80"/>
+      <x:c r="F6" s="80"/>
+      <x:c r="G6" s="80"/>
+      <x:c r="H6" s="81"/>
+    </x:row>
+    <x:row r="7" ht="30" customHeight="1">
+      <x:c r="A7" s="82"/>
+      <x:c r="B7" s="83"/>
+      <x:c r="C7" s="83"/>
+      <x:c r="D7" s="83"/>
+      <x:c r="E7" s="83"/>
+      <x:c r="F7" s="83"/>
+      <x:c r="G7" s="83"/>
+      <x:c r="H7" s="84"/>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="72" t="str">
+        <x:v>1 · Lock the baseline</x:v>
+      </x:c>
+      <x:c r="B9" s="73"/>
+      <x:c r="C9" s="73"/>
+      <x:c r="D9" s="73"/>
+      <x:c r="E9" s="73"/>
+      <x:c r="F9" s="73"/>
+      <x:c r="G9" s="73"/>
+      <x:c r="H9" s="74"/>
+    </x:row>
+    <x:row r="10" ht="30" customHeight="1">
+      <x:c r="A10" s="79" t="str">
+        <x:v>Before receiving the Scenario Reveal, submit the baseline allocation, IPS scorecard, and initial results through the designated Canvas checkpoint. Do not alter the submitted baseline after the reveal.</x:v>
+      </x:c>
+      <x:c r="B10" s="80"/>
+      <x:c r="C10" s="80"/>
+      <x:c r="D10" s="80"/>
+      <x:c r="E10" s="80"/>
+      <x:c r="F10" s="80"/>
+      <x:c r="G10" s="80"/>
+      <x:c r="H10" s="81"/>
+    </x:row>
+    <x:row r="11" ht="30" customHeight="1">
+      <x:c r="A11" s="82"/>
+      <x:c r="B11" s="83"/>
+      <x:c r="C11" s="83"/>
+      <x:c r="D11" s="83"/>
+      <x:c r="E11" s="83"/>
+      <x:c r="F11" s="83"/>
+      <x:c r="G11" s="83"/>
+      <x:c r="H11" s="84"/>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="72" t="str">
+        <x:v>2 · Record the instructor release</x:v>
+      </x:c>
+      <x:c r="B13" s="73"/>
+      <x:c r="C13" s="73"/>
+      <x:c r="D13" s="73"/>
+      <x:c r="E13" s="73"/>
+      <x:c r="F13" s="73"/>
+      <x:c r="G13" s="73"/>
+      <x:c r="H13" s="74"/>
+    </x:row>
+    <x:row r="14" ht="30" customHeight="1">
+      <x:c r="A14" s="79" t="str">
+        <x:v>Enter the packet identifier, release date, and the exact scenario inputs or event facts supplied by the instructor. Do not soften the inputs, change the client mandate, or invent values not in the packet.</x:v>
+      </x:c>
+      <x:c r="B14" s="80"/>
+      <x:c r="C14" s="80"/>
+      <x:c r="D14" s="80"/>
+      <x:c r="E14" s="80"/>
+      <x:c r="F14" s="80"/>
+      <x:c r="G14" s="80"/>
+      <x:c r="H14" s="81"/>
+    </x:row>
+    <x:row r="15" ht="30" customHeight="1">
+      <x:c r="A15" s="82"/>
+      <x:c r="B15" s="83"/>
+      <x:c r="C15" s="83"/>
+      <x:c r="D15" s="83"/>
+      <x:c r="E15" s="83"/>
+      <x:c r="F15" s="83"/>
+      <x:c r="G15" s="83"/>
+      <x:c r="H15" s="84"/>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="72" t="str">
+        <x:v>3 · Run the revealed scenario</x:v>
+      </x:c>
+      <x:c r="B17" s="73"/>
+      <x:c r="C17" s="73"/>
+      <x:c r="D17" s="73"/>
+      <x:c r="E17" s="73"/>
+      <x:c r="F17" s="73"/>
+      <x:c r="G17" s="73"/>
+      <x:c r="H17" s="74"/>
+    </x:row>
+    <x:row r="18" ht="30" customHeight="1">
+      <x:c r="A18" s="79" t="str">
+        <x:v>Transfer the released assumptions to the relevant Client tab, calculate the percentage and dollar impact, identify the exposed client goal or constraint, and record the result as Pass, Warning, or Breach.</x:v>
+      </x:c>
+      <x:c r="B18" s="80"/>
+      <x:c r="C18" s="80"/>
+      <x:c r="D18" s="80"/>
+      <x:c r="E18" s="80"/>
+      <x:c r="F18" s="80"/>
+      <x:c r="G18" s="80"/>
+      <x:c r="H18" s="81"/>
+    </x:row>
+    <x:row r="19" ht="30" customHeight="1">
+      <x:c r="A19" s="82"/>
+      <x:c r="B19" s="83"/>
+      <x:c r="C19" s="83"/>
+      <x:c r="D19" s="83"/>
+      <x:c r="E19" s="83"/>
+      <x:c r="F19" s="83"/>
+      <x:c r="G19" s="83"/>
+      <x:c r="H19" s="84"/>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="72" t="str">
+        <x:v>4 · Remediate and re-test</x:v>
+      </x:c>
+      <x:c r="B21" s="73"/>
+      <x:c r="C21" s="73"/>
+      <x:c r="D21" s="73"/>
+      <x:c r="E21" s="73"/>
+      <x:c r="F21" s="73"/>
+      <x:c r="G21" s="73"/>
+      <x:c r="H21" s="74"/>
+    </x:row>
+    <x:row r="22" ht="30" customHeight="1">
+      <x:c r="A22" s="79" t="str">
+        <x:v>A quantitative breach requires a real security, sleeve, or weight change. State the trade-off, re-run the full scenario and IPS tests, and retain both the baseline and revised evidence for Gate 2.</x:v>
+      </x:c>
+      <x:c r="B22" s="80"/>
+      <x:c r="C22" s="80"/>
+      <x:c r="D22" s="80"/>
+      <x:c r="E22" s="80"/>
+      <x:c r="F22" s="80"/>
+      <x:c r="G22" s="80"/>
+      <x:c r="H22" s="81"/>
+    </x:row>
+    <x:row r="23" ht="30" customHeight="1">
+      <x:c r="A23" s="82"/>
+      <x:c r="B23" s="83"/>
+      <x:c r="C23" s="83"/>
+      <x:c r="D23" s="83"/>
+      <x:c r="E23" s="83"/>
+      <x:c r="F23" s="83"/>
+      <x:c r="G23" s="83"/>
+      <x:c r="H23" s="84"/>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="72" t="str">
+        <x:v>Scenario Release Log — Complete after the instructor releases the packet</x:v>
+      </x:c>
+      <x:c r="B25" s="73"/>
+      <x:c r="C25" s="73"/>
+      <x:c r="D25" s="73"/>
+      <x:c r="E25" s="73"/>
+      <x:c r="F25" s="73"/>
+      <x:c r="G25" s="73"/>
+      <x:c r="H25" s="74"/>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="91" t="str">
+        <x:v>Client</x:v>
+      </x:c>
+      <x:c r="B26" s="91" t="str">
+        <x:v>Packet ID</x:v>
+      </x:c>
+      <x:c r="C26" s="91" t="str">
+        <x:v>Release date</x:v>
+      </x:c>
+      <x:c r="D26" s="91" t="str">
+        <x:v>Named client goal / constraint tested</x:v>
+      </x:c>
+      <x:c r="E26" s="91" t="str">
+        <x:v>Scenario inputs or event facts</x:v>
+      </x:c>
+      <x:c r="F26" s="91" t="str">
+        <x:v>Baseline receipt / submission confirmation</x:v>
+      </x:c>
+      <x:c r="G26" s="91" t="str">
+        <x:v>Initial result</x:v>
+      </x:c>
+      <x:c r="H26" s="91" t="str">
+        <x:v>Instructor follow-up if result is Pass</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="42" customHeight="1">
+      <x:c r="A27" s="93" t="str">
+        <x:v>Client 1</x:v>
+      </x:c>
+      <x:c r="B27" s="93" t="str"/>
+      <x:c r="C27" s="93" t="str"/>
+      <x:c r="D27" s="93" t="str"/>
+      <x:c r="E27" s="93" t="str"/>
+      <x:c r="F27" s="93" t="str"/>
+      <x:c r="G27" s="93" t="str"/>
+      <x:c r="H27" s="93" t="str"/>
+    </x:row>
+    <x:row r="28" ht="42" customHeight="1">
+      <x:c r="A28" s="93" t="str">
+        <x:v>Client 2</x:v>
+      </x:c>
+      <x:c r="B28" s="93" t="str"/>
+      <x:c r="C28" s="93" t="str"/>
+      <x:c r="D28" s="93" t="str"/>
+      <x:c r="E28" s="93" t="str"/>
+      <x:c r="F28" s="93" t="str"/>
+      <x:c r="G28" s="93" t="str"/>
+      <x:c r="H28" s="93" t="str"/>
+    </x:row>
+    <x:row r="29" ht="42" customHeight="1">
+      <x:c r="A29" s="93" t="str">
+        <x:v>Client 3</x:v>
+      </x:c>
+      <x:c r="B29" s="93" t="str"/>
+      <x:c r="C29" s="93" t="str"/>
+      <x:c r="D29" s="93" t="str"/>
+      <x:c r="E29" s="93" t="str"/>
+      <x:c r="F29" s="93" t="str"/>
+      <x:c r="G29" s="93" t="str"/>
+      <x:c r="H29" s="93" t="str"/>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="72" t="str">
+        <x:v>Required response rule</x:v>
+      </x:c>
+      <x:c r="B32" s="73"/>
+      <x:c r="C32" s="73"/>
+      <x:c r="D32" s="73"/>
+      <x:c r="E32" s="73"/>
+      <x:c r="F32" s="73"/>
+      <x:c r="G32" s="73"/>
+      <x:c r="H32" s="74"/>
+    </x:row>
+    <x:row r="33" ht="34" customHeight="1">
+      <x:c r="A33" s="79" t="str">
+        <x:v>Do not use a pre-hedged baseline or revised assumptions to avoid the exercise. If the revealed scenario shows a Breach, complete the trade log and revised test in the matching Client tab. If it unexpectedly shows Pass, stop and report the result to the instructor; do not treat a Pass as permission to skip the remediation checkpoint.</x:v>
+      </x:c>
+      <x:c r="B33" s="80"/>
+      <x:c r="C33" s="80"/>
+      <x:c r="D33" s="80"/>
+      <x:c r="E33" s="80"/>
+      <x:c r="F33" s="80"/>
+      <x:c r="G33" s="80"/>
+      <x:c r="H33" s="81"/>
+    </x:row>
+    <x:row r="34" ht="34" customHeight="1">
+      <x:c r="A34" s="94"/>
+      <x:c r="B34" s="95"/>
+      <x:c r="C34" s="95"/>
+      <x:c r="D34" s="95"/>
+      <x:c r="E34" s="95"/>
+      <x:c r="F34" s="95"/>
+      <x:c r="G34" s="95"/>
+      <x:c r="H34" s="96"/>
+    </x:row>
+    <x:row r="35" ht="34" customHeight="1">
+      <x:c r="A35" s="82"/>
+      <x:c r="B35" s="83"/>
+      <x:c r="C35" s="83"/>
+      <x:c r="D35" s="83"/>
+      <x:c r="E35" s="83"/>
+      <x:c r="F35" s="83"/>
+      <x:c r="G35" s="83"/>
+      <x:c r="H35" s="84"/>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:H1"/>
+    <x:mergeCell ref="A2:H2"/>
+    <x:mergeCell ref="A5:H5"/>
+    <x:mergeCell ref="A6:H7"/>
+    <x:mergeCell ref="A9:H9"/>
+    <x:mergeCell ref="A10:H11"/>
+    <x:mergeCell ref="A13:H13"/>
+    <x:mergeCell ref="A14:H15"/>
+    <x:mergeCell ref="A17:H17"/>
+    <x:mergeCell ref="A18:H19"/>
+    <x:mergeCell ref="A21:H21"/>
+    <x:mergeCell ref="A22:H23"/>
+    <x:mergeCell ref="A25:H25"/>
+    <x:mergeCell ref="A32:H32"/>
+    <x:mergeCell ref="A33:H35"/>
+  </x:mergeCells>
+  <x:dataValidations count="1">
+    <x:dataValidation type="list" sqref="G27:G29">
+      <x:formula1>"Pass,Warning,Breach"</x:formula1>
+    </x:dataValidation>
+  </x:dataValidations>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
</xml_diff>